<commit_message>
Proportionally scale net weight to match PL exact total
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -673,7 +673,7 @@
       <c r="H6" s="6" t="inlineStr"/>
       <c r="I6" s="6" t="inlineStr"/>
       <c r="J6" s="5" t="n">
-        <v>239.943</v>
+        <v>235.785</v>
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
@@ -696,16 +696,16 @@
         </is>
       </c>
       <c r="O6" s="5" t="n">
-        <v>178.47</v>
+        <v>175.377</v>
       </c>
       <c r="P6" s="5" t="n">
-        <v>198.3</v>
+        <v>194.863</v>
       </c>
       <c r="Q6" s="5" t="n">
-        <v>198.3</v>
+        <v>194.863</v>
       </c>
       <c r="R6" s="5" t="n">
-        <v>19.83</v>
+        <v>19.486</v>
       </c>
       <c r="S6" s="6" t="inlineStr"/>
       <c r="T6" s="6" t="inlineStr">
@@ -716,7 +716,7 @@
       <c r="U6" s="6" t="inlineStr"/>
       <c r="V6" s="6" t="inlineStr"/>
       <c r="W6" s="5" t="n">
-        <v>198.3</v>
+        <v>194.863</v>
       </c>
     </row>
     <row r="7">
@@ -740,7 +740,7 @@
       <c r="H7" s="6" t="inlineStr"/>
       <c r="I7" s="6" t="inlineStr"/>
       <c r="J7" s="5" t="n">
-        <v>8.349</v>
+        <v>8.204000000000001</v>
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
@@ -763,16 +763,16 @@
         </is>
       </c>
       <c r="O7" s="5" t="n">
-        <v>6.21</v>
+        <v>6.102</v>
       </c>
       <c r="P7" s="5" t="n">
-        <v>6.9</v>
+        <v>6.78</v>
       </c>
       <c r="Q7" s="5" t="n">
-        <v>6.9</v>
+        <v>6.78</v>
       </c>
       <c r="R7" s="5" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.678</v>
       </c>
       <c r="S7" s="6" t="inlineStr"/>
       <c r="T7" s="6" t="inlineStr">
@@ -783,7 +783,7 @@
       <c r="U7" s="6" t="inlineStr"/>
       <c r="V7" s="6" t="inlineStr"/>
       <c r="W7" s="5" t="n">
-        <v>6.9</v>
+        <v>6.78</v>
       </c>
     </row>
     <row r="8">
@@ -807,7 +807,7 @@
       <c r="H8" s="6" t="inlineStr"/>
       <c r="I8" s="6" t="inlineStr"/>
       <c r="J8" s="5" t="n">
-        <v>45.593</v>
+        <v>44.803</v>
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
@@ -830,16 +830,16 @@
         </is>
       </c>
       <c r="O8" s="5" t="n">
-        <v>33.912</v>
+        <v>33.324</v>
       </c>
       <c r="P8" s="5" t="n">
-        <v>37.68</v>
+        <v>37.027</v>
       </c>
       <c r="Q8" s="5" t="n">
-        <v>37.68</v>
+        <v>37.027</v>
       </c>
       <c r="R8" s="5" t="n">
-        <v>3.768</v>
+        <v>3.703</v>
       </c>
       <c r="S8" s="6" t="inlineStr"/>
       <c r="T8" s="6" t="inlineStr">
@@ -850,7 +850,7 @@
       <c r="U8" s="6" t="inlineStr"/>
       <c r="V8" s="6" t="inlineStr"/>
       <c r="W8" s="5" t="n">
-        <v>37.68</v>
+        <v>37.027</v>
       </c>
     </row>
     <row r="9">
@@ -874,7 +874,7 @@
       <c r="H9" s="6" t="inlineStr"/>
       <c r="I9" s="6" t="inlineStr"/>
       <c r="J9" s="5" t="n">
-        <v>50.215</v>
+        <v>49.345</v>
       </c>
       <c r="K9" s="6" t="inlineStr">
         <is>
@@ -897,16 +897,16 @@
         </is>
       </c>
       <c r="O9" s="5" t="n">
-        <v>37.35</v>
+        <v>36.703</v>
       </c>
       <c r="P9" s="5" t="n">
-        <v>41.5</v>
+        <v>40.781</v>
       </c>
       <c r="Q9" s="5" t="n">
-        <v>41.5</v>
+        <v>40.781</v>
       </c>
       <c r="R9" s="5" t="n">
-        <v>4.15</v>
+        <v>4.078</v>
       </c>
       <c r="S9" s="6" t="inlineStr"/>
       <c r="T9" s="6" t="inlineStr">
@@ -917,7 +917,7 @@
       <c r="U9" s="6" t="inlineStr"/>
       <c r="V9" s="6" t="inlineStr"/>
       <c r="W9" s="5" t="n">
-        <v>41.5</v>
+        <v>40.781</v>
       </c>
     </row>
     <row r="10">
@@ -941,7 +941,7 @@
       <c r="H10" s="6" t="inlineStr"/>
       <c r="I10" s="6" t="inlineStr"/>
       <c r="J10" s="5" t="n">
-        <v>69.45399999999999</v>
+        <v>68.25</v>
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
@@ -964,16 +964,16 @@
         </is>
       </c>
       <c r="O10" s="5" t="n">
-        <v>51.66</v>
+        <v>50.765</v>
       </c>
       <c r="P10" s="5" t="n">
-        <v>57.4</v>
+        <v>56.405</v>
       </c>
       <c r="Q10" s="5" t="n">
-        <v>57.4</v>
+        <v>56.405</v>
       </c>
       <c r="R10" s="5" t="n">
-        <v>5.74</v>
+        <v>5.641</v>
       </c>
       <c r="S10" s="6" t="inlineStr"/>
       <c r="T10" s="6" t="inlineStr">
@@ -984,7 +984,7 @@
       <c r="U10" s="6" t="inlineStr"/>
       <c r="V10" s="6" t="inlineStr"/>
       <c r="W10" s="5" t="n">
-        <v>57.4</v>
+        <v>56.405</v>
       </c>
     </row>
     <row r="11">
@@ -1008,7 +1008,7 @@
       <c r="H11" s="6" t="inlineStr"/>
       <c r="I11" s="6" t="inlineStr"/>
       <c r="J11" s="5" t="n">
-        <v>31</v>
+        <v>30.463</v>
       </c>
       <c r="K11" s="6" t="inlineStr">
         <is>
@@ -1031,16 +1031,16 @@
         </is>
       </c>
       <c r="O11" s="5" t="n">
-        <v>23.058</v>
+        <v>22.658</v>
       </c>
       <c r="P11" s="5" t="n">
-        <v>25.62</v>
+        <v>25.176</v>
       </c>
       <c r="Q11" s="5" t="n">
-        <v>25.62</v>
+        <v>25.176</v>
       </c>
       <c r="R11" s="5" t="n">
-        <v>2.562</v>
+        <v>2.518</v>
       </c>
       <c r="S11" s="6" t="inlineStr"/>
       <c r="T11" s="6" t="inlineStr">
@@ -1051,7 +1051,7 @@
       <c r="U11" s="6" t="inlineStr"/>
       <c r="V11" s="6" t="inlineStr"/>
       <c r="W11" s="5" t="n">
-        <v>25.62</v>
+        <v>25.176</v>
       </c>
     </row>
     <row r="12">
@@ -1075,7 +1075,7 @@
       <c r="H12" s="6" t="inlineStr"/>
       <c r="I12" s="6" t="inlineStr"/>
       <c r="J12" s="5" t="n">
-        <v>46.27</v>
+        <v>45.469</v>
       </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
@@ -1098,16 +1098,16 @@
         </is>
       </c>
       <c r="O12" s="5" t="n">
-        <v>34.416</v>
+        <v>33.82</v>
       </c>
       <c r="P12" s="5" t="n">
-        <v>38.24</v>
+        <v>37.577</v>
       </c>
       <c r="Q12" s="5" t="n">
-        <v>38.24</v>
+        <v>37.577</v>
       </c>
       <c r="R12" s="5" t="n">
-        <v>3.824</v>
+        <v>3.758</v>
       </c>
       <c r="S12" s="6" t="inlineStr"/>
       <c r="T12" s="6" t="inlineStr">
@@ -1118,7 +1118,7 @@
       <c r="U12" s="6" t="inlineStr"/>
       <c r="V12" s="6" t="inlineStr"/>
       <c r="W12" s="5" t="n">
-        <v>38.24</v>
+        <v>37.577</v>
       </c>
     </row>
     <row r="13">
@@ -1142,7 +1142,7 @@
       <c r="H13" s="6" t="inlineStr"/>
       <c r="I13" s="6" t="inlineStr"/>
       <c r="J13" s="5" t="n">
-        <v>27.298</v>
+        <v>26.825</v>
       </c>
       <c r="K13" s="6" t="inlineStr">
         <is>
@@ -1165,16 +1165,16 @@
         </is>
       </c>
       <c r="O13" s="5" t="n">
-        <v>20.304</v>
+        <v>19.952</v>
       </c>
       <c r="P13" s="5" t="n">
-        <v>22.56</v>
+        <v>22.169</v>
       </c>
       <c r="Q13" s="5" t="n">
-        <v>22.56</v>
+        <v>22.169</v>
       </c>
       <c r="R13" s="5" t="n">
-        <v>2.256</v>
+        <v>2.217</v>
       </c>
       <c r="S13" s="6" t="inlineStr"/>
       <c r="T13" s="6" t="inlineStr">
@@ -1185,7 +1185,7 @@
       <c r="U13" s="6" t="inlineStr"/>
       <c r="V13" s="6" t="inlineStr"/>
       <c r="W13" s="5" t="n">
-        <v>22.56</v>
+        <v>22.169</v>
       </c>
     </row>
     <row r="14">
@@ -1209,7 +1209,7 @@
       <c r="H14" s="6" t="inlineStr"/>
       <c r="I14" s="6" t="inlineStr"/>
       <c r="J14" s="5" t="n">
-        <v>138.739</v>
+        <v>136.334</v>
       </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
@@ -1232,16 +1232,16 @@
         </is>
       </c>
       <c r="O14" s="5" t="n">
-        <v>103.194</v>
+        <v>101.406</v>
       </c>
       <c r="P14" s="5" t="n">
-        <v>114.66</v>
+        <v>112.673</v>
       </c>
       <c r="Q14" s="5" t="n">
-        <v>114.66</v>
+        <v>112.673</v>
       </c>
       <c r="R14" s="5" t="n">
-        <v>11.466</v>
+        <v>11.267</v>
       </c>
       <c r="S14" s="6" t="inlineStr"/>
       <c r="T14" s="6" t="inlineStr">
@@ -1252,7 +1252,7 @@
       <c r="U14" s="6" t="inlineStr"/>
       <c r="V14" s="6" t="inlineStr"/>
       <c r="W14" s="5" t="n">
-        <v>114.66</v>
+        <v>112.673</v>
       </c>
     </row>
     <row r="15">
@@ -1276,7 +1276,7 @@
       <c r="H15" s="6" t="inlineStr"/>
       <c r="I15" s="6" t="inlineStr"/>
       <c r="J15" s="5" t="n">
-        <v>7.26</v>
+        <v>7.134</v>
       </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
@@ -1299,16 +1299,16 @@
         </is>
       </c>
       <c r="O15" s="5" t="n">
-        <v>5.4</v>
+        <v>5.306</v>
       </c>
       <c r="P15" s="5" t="n">
-        <v>6</v>
+        <v>5.896</v>
       </c>
       <c r="Q15" s="5" t="n">
-        <v>6</v>
+        <v>5.896</v>
       </c>
       <c r="R15" s="5" t="n">
-        <v>0.6</v>
+        <v>0.59</v>
       </c>
       <c r="S15" s="6" t="inlineStr"/>
       <c r="T15" s="6" t="inlineStr">
@@ -1319,7 +1319,7 @@
       <c r="U15" s="6" t="inlineStr"/>
       <c r="V15" s="6" t="inlineStr"/>
       <c r="W15" s="5" t="n">
-        <v>6</v>
+        <v>5.896</v>
       </c>
     </row>
     <row r="16">
@@ -1343,7 +1343,7 @@
       <c r="H16" s="6" t="inlineStr"/>
       <c r="I16" s="6" t="inlineStr"/>
       <c r="J16" s="5" t="n">
-        <v>347.754</v>
+        <v>341.727</v>
       </c>
       <c r="K16" s="6" t="inlineStr">
         <is>
@@ -1366,16 +1366,16 @@
         </is>
       </c>
       <c r="O16" s="5" t="n">
-        <v>258.66</v>
+        <v>254.177</v>
       </c>
       <c r="P16" s="5" t="n">
-        <v>287.4</v>
+        <v>282.419</v>
       </c>
       <c r="Q16" s="5" t="n">
-        <v>287.4</v>
+        <v>282.419</v>
       </c>
       <c r="R16" s="5" t="n">
-        <v>28.74</v>
+        <v>28.242</v>
       </c>
       <c r="S16" s="6" t="inlineStr"/>
       <c r="T16" s="6" t="inlineStr">
@@ -1386,7 +1386,7 @@
       <c r="U16" s="6" t="inlineStr"/>
       <c r="V16" s="6" t="inlineStr"/>
       <c r="W16" s="5" t="n">
-        <v>287.4</v>
+        <v>282.419</v>
       </c>
     </row>
     <row r="17">
@@ -1410,7 +1410,7 @@
       <c r="H17" s="6" t="inlineStr"/>
       <c r="I17" s="6" t="inlineStr"/>
       <c r="J17" s="5" t="n">
-        <v>2.468</v>
+        <v>2.426</v>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
@@ -1433,16 +1433,16 @@
         </is>
       </c>
       <c r="O17" s="5" t="n">
-        <v>1.836</v>
+        <v>1.804</v>
       </c>
       <c r="P17" s="5" t="n">
-        <v>2.04</v>
+        <v>2.005</v>
       </c>
       <c r="Q17" s="5" t="n">
-        <v>2.04</v>
+        <v>2.005</v>
       </c>
       <c r="R17" s="5" t="n">
-        <v>0.204</v>
+        <v>0.2</v>
       </c>
       <c r="S17" s="6" t="inlineStr"/>
       <c r="T17" s="6" t="inlineStr">
@@ -1453,7 +1453,7 @@
       <c r="U17" s="6" t="inlineStr"/>
       <c r="V17" s="6" t="inlineStr"/>
       <c r="W17" s="5" t="n">
-        <v>2.04</v>
+        <v>2.005</v>
       </c>
     </row>
     <row r="18">
@@ -1477,7 +1477,7 @@
       <c r="H18" s="6" t="inlineStr"/>
       <c r="I18" s="6" t="inlineStr"/>
       <c r="J18" s="5" t="n">
-        <v>167.827</v>
+        <v>164.918</v>
       </c>
       <c r="K18" s="6" t="inlineStr">
         <is>
@@ -1500,16 +1500,16 @@
         </is>
       </c>
       <c r="O18" s="5" t="n">
-        <v>124.83</v>
+        <v>122.667</v>
       </c>
       <c r="P18" s="5" t="n">
-        <v>138.7</v>
+        <v>136.296</v>
       </c>
       <c r="Q18" s="5" t="n">
-        <v>138.7</v>
+        <v>136.296</v>
       </c>
       <c r="R18" s="5" t="n">
-        <v>13.87</v>
+        <v>13.63</v>
       </c>
       <c r="S18" s="6" t="inlineStr"/>
       <c r="T18" s="6" t="inlineStr">
@@ -1520,7 +1520,7 @@
       <c r="U18" s="6" t="inlineStr"/>
       <c r="V18" s="6" t="inlineStr"/>
       <c r="W18" s="5" t="n">
-        <v>138.7</v>
+        <v>136.296</v>
       </c>
     </row>
     <row r="19">
@@ -1544,7 +1544,7 @@
       <c r="H19" s="6" t="inlineStr"/>
       <c r="I19" s="6" t="inlineStr"/>
       <c r="J19" s="5" t="n">
-        <v>107.738</v>
+        <v>105.871</v>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
@@ -1567,16 +1567,16 @@
         </is>
       </c>
       <c r="O19" s="5" t="n">
-        <v>80.136</v>
+        <v>78.747</v>
       </c>
       <c r="P19" s="5" t="n">
-        <v>89.04000000000001</v>
+        <v>87.497</v>
       </c>
       <c r="Q19" s="5" t="n">
-        <v>89.04000000000001</v>
+        <v>87.497</v>
       </c>
       <c r="R19" s="5" t="n">
-        <v>8.904</v>
+        <v>8.75</v>
       </c>
       <c r="S19" s="6" t="inlineStr"/>
       <c r="T19" s="6" t="inlineStr">
@@ -1587,7 +1587,7 @@
       <c r="U19" s="6" t="inlineStr"/>
       <c r="V19" s="6" t="inlineStr"/>
       <c r="W19" s="5" t="n">
-        <v>89.04000000000001</v>
+        <v>87.497</v>
       </c>
     </row>
     <row r="20">
@@ -1611,7 +1611,7 @@
       <c r="H20" s="6" t="inlineStr"/>
       <c r="I20" s="6" t="inlineStr"/>
       <c r="J20" s="5" t="n">
-        <v>147.705</v>
+        <v>145.145</v>
       </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
@@ -1634,16 +1634,16 @@
         </is>
       </c>
       <c r="O20" s="5" t="n">
-        <v>109.863</v>
+        <v>107.959</v>
       </c>
       <c r="P20" s="5" t="n">
-        <v>122.07</v>
+        <v>119.954</v>
       </c>
       <c r="Q20" s="5" t="n">
-        <v>122.07</v>
+        <v>119.954</v>
       </c>
       <c r="R20" s="5" t="n">
-        <v>12.207</v>
+        <v>11.995</v>
       </c>
       <c r="S20" s="6" t="inlineStr"/>
       <c r="T20" s="6" t="inlineStr">
@@ -1654,7 +1654,7 @@
       <c r="U20" s="6" t="inlineStr"/>
       <c r="V20" s="6" t="inlineStr"/>
       <c r="W20" s="5" t="n">
-        <v>122.07</v>
+        <v>119.954</v>
       </c>
     </row>
     <row r="21">
@@ -1678,7 +1678,7 @@
       <c r="H21" s="6" t="inlineStr"/>
       <c r="I21" s="6" t="inlineStr"/>
       <c r="J21" s="5" t="n">
-        <v>84.869</v>
+        <v>83.399</v>
       </c>
       <c r="K21" s="6" t="inlineStr">
         <is>
@@ -1701,16 +1701,16 @@
         </is>
       </c>
       <c r="O21" s="5" t="n">
-        <v>63.126</v>
+        <v>62.032</v>
       </c>
       <c r="P21" s="5" t="n">
-        <v>70.14</v>
+        <v>68.92400000000001</v>
       </c>
       <c r="Q21" s="5" t="n">
-        <v>70.14</v>
+        <v>68.92400000000001</v>
       </c>
       <c r="R21" s="5" t="n">
-        <v>7.014</v>
+        <v>6.892</v>
       </c>
       <c r="S21" s="6" t="inlineStr"/>
       <c r="T21" s="6" t="inlineStr">
@@ -1721,7 +1721,7 @@
       <c r="U21" s="6" t="inlineStr"/>
       <c r="V21" s="6" t="inlineStr"/>
       <c r="W21" s="5" t="n">
-        <v>70.14</v>
+        <v>68.92400000000001</v>
       </c>
     </row>
     <row r="22">
@@ -1745,7 +1745,7 @@
       <c r="H22" s="6" t="inlineStr"/>
       <c r="I22" s="6" t="inlineStr"/>
       <c r="J22" s="5" t="n">
-        <v>77.92400000000001</v>
+        <v>76.574</v>
       </c>
       <c r="K22" s="6" t="inlineStr">
         <is>
@@ -1768,16 +1768,16 @@
         </is>
       </c>
       <c r="O22" s="5" t="n">
-        <v>57.96</v>
+        <v>56.956</v>
       </c>
       <c r="P22" s="5" t="n">
-        <v>64.40000000000001</v>
+        <v>63.284</v>
       </c>
       <c r="Q22" s="5" t="n">
-        <v>64.40000000000001</v>
+        <v>63.284</v>
       </c>
       <c r="R22" s="5" t="n">
-        <v>6.44</v>
+        <v>6.328</v>
       </c>
       <c r="S22" s="6" t="inlineStr"/>
       <c r="T22" s="6" t="inlineStr">
@@ -1788,7 +1788,7 @@
       <c r="U22" s="6" t="inlineStr"/>
       <c r="V22" s="6" t="inlineStr"/>
       <c r="W22" s="5" t="n">
-        <v>64.40000000000001</v>
+        <v>63.284</v>
       </c>
     </row>
     <row r="23">
@@ -1812,7 +1812,7 @@
       <c r="H23" s="6" t="inlineStr"/>
       <c r="I23" s="6" t="inlineStr"/>
       <c r="J23" s="5" t="n">
-        <v>122.513</v>
+        <v>120.389</v>
       </c>
       <c r="K23" s="6" t="inlineStr">
         <is>
@@ -1835,16 +1835,16 @@
         </is>
       </c>
       <c r="O23" s="5" t="n">
-        <v>91.125</v>
+        <v>89.54600000000001</v>
       </c>
       <c r="P23" s="5" t="n">
-        <v>101.25</v>
+        <v>99.495</v>
       </c>
       <c r="Q23" s="5" t="n">
-        <v>101.25</v>
+        <v>99.495</v>
       </c>
       <c r="R23" s="5" t="n">
-        <v>10.125</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="S23" s="6" t="inlineStr"/>
       <c r="T23" s="6" t="inlineStr">
@@ -1855,7 +1855,7 @@
       <c r="U23" s="6" t="inlineStr"/>
       <c r="V23" s="6" t="inlineStr"/>
       <c r="W23" s="5" t="n">
-        <v>101.25</v>
+        <v>99.495</v>
       </c>
     </row>
     <row r="24">
@@ -1879,7 +1879,7 @@
       <c r="H24" s="6" t="inlineStr"/>
       <c r="I24" s="6" t="inlineStr"/>
       <c r="J24" s="5" t="n">
-        <v>1.21</v>
+        <v>1.189</v>
       </c>
       <c r="K24" s="6" t="inlineStr">
         <is>
@@ -1902,16 +1902,16 @@
         </is>
       </c>
       <c r="O24" s="5" t="n">
-        <v>0.9</v>
+        <v>0.884</v>
       </c>
       <c r="P24" s="5" t="n">
-        <v>1</v>
+        <v>0.983</v>
       </c>
       <c r="Q24" s="5" t="n">
-        <v>1</v>
+        <v>0.983</v>
       </c>
       <c r="R24" s="5" t="n">
-        <v>0.1</v>
+        <v>0.098</v>
       </c>
       <c r="S24" s="6" t="inlineStr"/>
       <c r="T24" s="6" t="inlineStr">
@@ -1922,7 +1922,7 @@
       <c r="U24" s="6" t="inlineStr"/>
       <c r="V24" s="6" t="inlineStr"/>
       <c r="W24" s="5" t="n">
-        <v>1</v>
+        <v>0.983</v>
       </c>
     </row>
     <row r="25">
@@ -1946,7 +1946,7 @@
       <c r="H25" s="6" t="inlineStr"/>
       <c r="I25" s="6" t="inlineStr"/>
       <c r="J25" s="5" t="n">
-        <v>265.958</v>
+        <v>130.674</v>
       </c>
       <c r="K25" s="6" t="inlineStr">
         <is>
@@ -1969,16 +1969,16 @@
         </is>
       </c>
       <c r="O25" s="5" t="n">
-        <v>197.82</v>
+        <v>97.196</v>
       </c>
       <c r="P25" s="5" t="n">
-        <v>219.8</v>
+        <v>107.995</v>
       </c>
       <c r="Q25" s="5" t="n">
-        <v>219.8</v>
+        <v>107.995</v>
       </c>
       <c r="R25" s="5" t="n">
-        <v>21.98</v>
+        <v>10.8</v>
       </c>
       <c r="S25" s="6" t="inlineStr"/>
       <c r="T25" s="6" t="inlineStr">
@@ -1989,7 +1989,7 @@
       <c r="U25" s="6" t="inlineStr"/>
       <c r="V25" s="6" t="inlineStr"/>
       <c r="W25" s="5" t="n">
-        <v>219.8</v>
+        <v>107.995</v>
       </c>
     </row>
     <row r="26">
@@ -2013,7 +2013,7 @@
       <c r="H26" s="6" t="inlineStr"/>
       <c r="I26" s="6" t="inlineStr"/>
       <c r="J26" s="5" t="n">
-        <v>2.783</v>
+        <v>2.735</v>
       </c>
       <c r="K26" s="6" t="inlineStr">
         <is>
@@ -2036,16 +2036,16 @@
         </is>
       </c>
       <c r="O26" s="5" t="n">
-        <v>2.07</v>
+        <v>2.034</v>
       </c>
       <c r="P26" s="5" t="n">
-        <v>2.3</v>
+        <v>2.26</v>
       </c>
       <c r="Q26" s="5" t="n">
-        <v>2.3</v>
+        <v>2.26</v>
       </c>
       <c r="R26" s="5" t="n">
-        <v>0.23</v>
+        <v>0.226</v>
       </c>
       <c r="S26" s="6" t="inlineStr"/>
       <c r="T26" s="6" t="inlineStr">
@@ -2056,7 +2056,7 @@
       <c r="U26" s="6" t="inlineStr"/>
       <c r="V26" s="6" t="inlineStr"/>
       <c r="W26" s="5" t="n">
-        <v>2.3</v>
+        <v>2.26</v>
       </c>
     </row>
     <row r="27">
@@ -2080,7 +2080,7 @@
       <c r="H27" s="6" t="inlineStr"/>
       <c r="I27" s="6" t="inlineStr"/>
       <c r="J27" s="5" t="n">
-        <v>123.057</v>
+        <v>120.924</v>
       </c>
       <c r="K27" s="6" t="inlineStr">
         <is>
@@ -2103,16 +2103,16 @@
         </is>
       </c>
       <c r="O27" s="5" t="n">
-        <v>91.53</v>
+        <v>89.944</v>
       </c>
       <c r="P27" s="5" t="n">
-        <v>101.7</v>
+        <v>99.937</v>
       </c>
       <c r="Q27" s="5" t="n">
-        <v>101.7</v>
+        <v>99.937</v>
       </c>
       <c r="R27" s="5" t="n">
-        <v>10.17</v>
+        <v>9.994</v>
       </c>
       <c r="S27" s="6" t="inlineStr"/>
       <c r="T27" s="6" t="inlineStr">
@@ -2123,7 +2123,7 @@
       <c r="U27" s="6" t="inlineStr"/>
       <c r="V27" s="6" t="inlineStr"/>
       <c r="W27" s="5" t="n">
-        <v>101.7</v>
+        <v>99.937</v>
       </c>
     </row>
     <row r="28">
@@ -2147,7 +2147,7 @@
       <c r="H28" s="6" t="inlineStr"/>
       <c r="I28" s="6" t="inlineStr"/>
       <c r="J28" s="5" t="n">
-        <v>2.904</v>
+        <v>2.854</v>
       </c>
       <c r="K28" s="6" t="inlineStr">
         <is>
@@ -2170,16 +2170,16 @@
         </is>
       </c>
       <c r="O28" s="5" t="n">
-        <v>2.16</v>
+        <v>2.123</v>
       </c>
       <c r="P28" s="5" t="n">
-        <v>2.4</v>
+        <v>2.358</v>
       </c>
       <c r="Q28" s="5" t="n">
-        <v>2.4</v>
+        <v>2.358</v>
       </c>
       <c r="R28" s="5" t="n">
-        <v>0.24</v>
+        <v>0.236</v>
       </c>
       <c r="S28" s="6" t="inlineStr"/>
       <c r="T28" s="6" t="inlineStr">
@@ -2190,7 +2190,7 @@
       <c r="U28" s="6" t="inlineStr"/>
       <c r="V28" s="6" t="inlineStr"/>
       <c r="W28" s="5" t="n">
-        <v>2.4</v>
+        <v>2.358</v>
       </c>
     </row>
     <row r="29">
@@ -2214,7 +2214,7 @@
       <c r="H29" s="6" t="inlineStr"/>
       <c r="I29" s="6" t="inlineStr"/>
       <c r="J29" s="5" t="n">
-        <v>6.389</v>
+        <v>6.278</v>
       </c>
       <c r="K29" s="6" t="inlineStr">
         <is>
@@ -2237,16 +2237,16 @@
         </is>
       </c>
       <c r="O29" s="5" t="n">
-        <v>4.752</v>
+        <v>4.67</v>
       </c>
       <c r="P29" s="5" t="n">
-        <v>5.28</v>
+        <v>5.188</v>
       </c>
       <c r="Q29" s="5" t="n">
-        <v>5.28</v>
+        <v>5.188</v>
       </c>
       <c r="R29" s="5" t="n">
-        <v>0.528</v>
+        <v>0.519</v>
       </c>
       <c r="S29" s="6" t="inlineStr"/>
       <c r="T29" s="6" t="inlineStr">
@@ -2257,7 +2257,7 @@
       <c r="U29" s="6" t="inlineStr"/>
       <c r="V29" s="6" t="inlineStr"/>
       <c r="W29" s="5" t="n">
-        <v>5.28</v>
+        <v>5.188</v>
       </c>
     </row>
     <row r="30">
@@ -2281,7 +2281,7 @@
       <c r="H30" s="6" t="inlineStr"/>
       <c r="I30" s="6" t="inlineStr"/>
       <c r="J30" s="5" t="n">
-        <v>20.703</v>
+        <v>20.344</v>
       </c>
       <c r="K30" s="6" t="inlineStr">
         <is>
@@ -2304,16 +2304,16 @@
         </is>
       </c>
       <c r="O30" s="5" t="n">
-        <v>15.399</v>
+        <v>15.132</v>
       </c>
       <c r="P30" s="5" t="n">
-        <v>17.11</v>
+        <v>16.813</v>
       </c>
       <c r="Q30" s="5" t="n">
-        <v>17.11</v>
+        <v>16.813</v>
       </c>
       <c r="R30" s="5" t="n">
-        <v>1.711</v>
+        <v>1.681</v>
       </c>
       <c r="S30" s="6" t="inlineStr"/>
       <c r="T30" s="6" t="inlineStr">
@@ -2324,7 +2324,7 @@
       <c r="U30" s="6" t="inlineStr"/>
       <c r="V30" s="6" t="inlineStr"/>
       <c r="W30" s="5" t="n">
-        <v>17.11</v>
+        <v>16.813</v>
       </c>
     </row>
     <row r="31">
@@ -2348,7 +2348,7 @@
       <c r="H31" s="6" t="inlineStr"/>
       <c r="I31" s="6" t="inlineStr"/>
       <c r="J31" s="5" t="n">
-        <v>10.164</v>
+        <v>9.988</v>
       </c>
       <c r="K31" s="6" t="inlineStr">
         <is>
@@ -2371,16 +2371,16 @@
         </is>
       </c>
       <c r="O31" s="5" t="n">
-        <v>7.56</v>
+        <v>7.429</v>
       </c>
       <c r="P31" s="5" t="n">
-        <v>8.4</v>
+        <v>8.254</v>
       </c>
       <c r="Q31" s="5" t="n">
-        <v>8.4</v>
+        <v>8.254</v>
       </c>
       <c r="R31" s="5" t="n">
-        <v>0.84</v>
+        <v>0.825</v>
       </c>
       <c r="S31" s="6" t="inlineStr"/>
       <c r="T31" s="6" t="inlineStr">
@@ -2391,7 +2391,7 @@
       <c r="U31" s="6" t="inlineStr"/>
       <c r="V31" s="6" t="inlineStr"/>
       <c r="W31" s="5" t="n">
-        <v>8.4</v>
+        <v>8.254</v>
       </c>
     </row>
     <row r="32">
@@ -2415,7 +2415,7 @@
       <c r="H32" s="6" t="inlineStr"/>
       <c r="I32" s="6" t="inlineStr"/>
       <c r="J32" s="5" t="n">
-        <v>5.082</v>
+        <v>3.995</v>
       </c>
       <c r="K32" s="6" t="inlineStr">
         <is>
@@ -2438,16 +2438,16 @@
         </is>
       </c>
       <c r="O32" s="5" t="n">
-        <v>3.78</v>
+        <v>2.972</v>
       </c>
       <c r="P32" s="5" t="n">
-        <v>4.2</v>
+        <v>3.302</v>
       </c>
       <c r="Q32" s="5" t="n">
-        <v>4.2</v>
+        <v>3.302</v>
       </c>
       <c r="R32" s="5" t="n">
-        <v>0.42</v>
+        <v>0.33</v>
       </c>
       <c r="S32" s="6" t="inlineStr"/>
       <c r="T32" s="6" t="inlineStr">
@@ -2458,7 +2458,7 @@
       <c r="U32" s="6" t="inlineStr"/>
       <c r="V32" s="6" t="inlineStr"/>
       <c r="W32" s="5" t="n">
-        <v>4.2</v>
+        <v>3.302</v>
       </c>
     </row>
     <row r="33">
@@ -2482,7 +2482,7 @@
       <c r="H33" s="6" t="inlineStr"/>
       <c r="I33" s="6" t="inlineStr"/>
       <c r="J33" s="5" t="n">
-        <v>12.342</v>
+        <v>9.702</v>
       </c>
       <c r="K33" s="6" t="inlineStr">
         <is>
@@ -2505,16 +2505,16 @@
         </is>
       </c>
       <c r="O33" s="5" t="n">
-        <v>9.18</v>
+        <v>7.217</v>
       </c>
       <c r="P33" s="5" t="n">
-        <v>10.2</v>
+        <v>8.019</v>
       </c>
       <c r="Q33" s="5" t="n">
-        <v>10.2</v>
+        <v>8.019</v>
       </c>
       <c r="R33" s="5" t="n">
-        <v>1.02</v>
+        <v>0.802</v>
       </c>
       <c r="S33" s="6" t="inlineStr"/>
       <c r="T33" s="6" t="inlineStr">
@@ -2525,7 +2525,7 @@
       <c r="U33" s="6" t="inlineStr"/>
       <c r="V33" s="6" t="inlineStr"/>
       <c r="W33" s="5" t="n">
-        <v>10.2</v>
+        <v>8.019</v>
       </c>
     </row>
     <row r="34">
@@ -2549,7 +2549,7 @@
       <c r="H34" s="6" t="inlineStr"/>
       <c r="I34" s="6" t="inlineStr"/>
       <c r="J34" s="5" t="n">
-        <v>22.506</v>
+        <v>13.27</v>
       </c>
       <c r="K34" s="6" t="inlineStr">
         <is>
@@ -2572,16 +2572,16 @@
         </is>
       </c>
       <c r="O34" s="5" t="n">
-        <v>16.74</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="P34" s="5" t="n">
-        <v>18.6</v>
+        <v>10.967</v>
       </c>
       <c r="Q34" s="5" t="n">
-        <v>18.6</v>
+        <v>10.967</v>
       </c>
       <c r="R34" s="5" t="n">
-        <v>1.86</v>
+        <v>1.097</v>
       </c>
       <c r="S34" s="6" t="inlineStr"/>
       <c r="T34" s="6" t="inlineStr">
@@ -2592,7 +2592,7 @@
       <c r="U34" s="6" t="inlineStr"/>
       <c r="V34" s="6" t="inlineStr"/>
       <c r="W34" s="5" t="n">
-        <v>18.6</v>
+        <v>10.967</v>
       </c>
     </row>
     <row r="35">
@@ -2616,7 +2616,7 @@
       <c r="H35" s="6" t="inlineStr"/>
       <c r="I35" s="6" t="inlineStr"/>
       <c r="J35" s="5" t="n">
-        <v>1.936</v>
+        <v>1.902</v>
       </c>
       <c r="K35" s="6" t="inlineStr">
         <is>
@@ -2639,16 +2639,16 @@
         </is>
       </c>
       <c r="O35" s="5" t="n">
-        <v>1.44</v>
+        <v>1.415</v>
       </c>
       <c r="P35" s="5" t="n">
-        <v>1.6</v>
+        <v>1.572</v>
       </c>
       <c r="Q35" s="5" t="n">
-        <v>1.6</v>
+        <v>1.572</v>
       </c>
       <c r="R35" s="5" t="n">
-        <v>0.16</v>
+        <v>0.157</v>
       </c>
       <c r="S35" s="6" t="inlineStr"/>
       <c r="T35" s="6" t="inlineStr">
@@ -2659,7 +2659,7 @@
       <c r="U35" s="6" t="inlineStr"/>
       <c r="V35" s="6" t="inlineStr"/>
       <c r="W35" s="5" t="n">
-        <v>1.6</v>
+        <v>1.572</v>
       </c>
     </row>
     <row r="36">
@@ -2683,7 +2683,7 @@
       <c r="H36" s="6" t="inlineStr"/>
       <c r="I36" s="6" t="inlineStr"/>
       <c r="J36" s="5" t="n">
-        <v>7.284</v>
+        <v>5.113</v>
       </c>
       <c r="K36" s="6" t="inlineStr">
         <is>
@@ -2706,16 +2706,16 @@
         </is>
       </c>
       <c r="O36" s="5" t="n">
-        <v>5.418</v>
+        <v>3.803</v>
       </c>
       <c r="P36" s="5" t="n">
-        <v>6.02</v>
+        <v>4.225</v>
       </c>
       <c r="Q36" s="5" t="n">
-        <v>6.02</v>
+        <v>4.225</v>
       </c>
       <c r="R36" s="5" t="n">
-        <v>0.602</v>
+        <v>0.423</v>
       </c>
       <c r="S36" s="6" t="inlineStr"/>
       <c r="T36" s="6" t="inlineStr">
@@ -2726,7 +2726,7 @@
       <c r="U36" s="6" t="inlineStr"/>
       <c r="V36" s="6" t="inlineStr"/>
       <c r="W36" s="5" t="n">
-        <v>6.02</v>
+        <v>4.225</v>
       </c>
     </row>
     <row r="37">
@@ -2750,7 +2750,7 @@
       <c r="H37" s="6" t="inlineStr"/>
       <c r="I37" s="6" t="inlineStr"/>
       <c r="J37" s="5" t="n">
-        <v>25.289</v>
+        <v>19.881</v>
       </c>
       <c r="K37" s="6" t="inlineStr">
         <is>
@@ -2773,16 +2773,16 @@
         </is>
       </c>
       <c r="O37" s="5" t="n">
-        <v>18.81</v>
+        <v>14.787</v>
       </c>
       <c r="P37" s="5" t="n">
-        <v>20.9</v>
+        <v>16.43</v>
       </c>
       <c r="Q37" s="5" t="n">
-        <v>20.9</v>
+        <v>16.43</v>
       </c>
       <c r="R37" s="5" t="n">
-        <v>2.09</v>
+        <v>1.643</v>
       </c>
       <c r="S37" s="6" t="inlineStr"/>
       <c r="T37" s="6" t="inlineStr">
@@ -2793,7 +2793,7 @@
       <c r="U37" s="6" t="inlineStr"/>
       <c r="V37" s="6" t="inlineStr"/>
       <c r="W37" s="5" t="n">
-        <v>20.9</v>
+        <v>16.43</v>
       </c>
     </row>
     <row r="38">
@@ -2817,7 +2817,7 @@
       <c r="H38" s="6" t="inlineStr"/>
       <c r="I38" s="6" t="inlineStr"/>
       <c r="J38" s="5" t="n">
-        <v>5.59</v>
+        <v>5.493</v>
       </c>
       <c r="K38" s="6" t="inlineStr">
         <is>
@@ -2840,16 +2840,16 @@
         </is>
       </c>
       <c r="O38" s="5" t="n">
-        <v>4.158</v>
+        <v>4.086</v>
       </c>
       <c r="P38" s="5" t="n">
-        <v>4.62</v>
+        <v>4.54</v>
       </c>
       <c r="Q38" s="5" t="n">
-        <v>4.62</v>
+        <v>4.54</v>
       </c>
       <c r="R38" s="5" t="n">
-        <v>0.462</v>
+        <v>0.454</v>
       </c>
       <c r="S38" s="6" t="inlineStr"/>
       <c r="T38" s="6" t="inlineStr">
@@ -2860,7 +2860,7 @@
       <c r="U38" s="6" t="inlineStr"/>
       <c r="V38" s="6" t="inlineStr"/>
       <c r="W38" s="5" t="n">
-        <v>4.62</v>
+        <v>4.54</v>
       </c>
     </row>
     <row r="39">
@@ -2884,7 +2884,7 @@
       <c r="H39" s="6" t="inlineStr"/>
       <c r="I39" s="6" t="inlineStr"/>
       <c r="J39" s="5" t="n">
-        <v>29.524</v>
+        <v>29.012</v>
       </c>
       <c r="K39" s="6" t="inlineStr">
         <is>
@@ -2907,16 +2907,16 @@
         </is>
       </c>
       <c r="O39" s="5" t="n">
-        <v>21.96</v>
+        <v>21.579</v>
       </c>
       <c r="P39" s="5" t="n">
-        <v>24.4</v>
+        <v>23.977</v>
       </c>
       <c r="Q39" s="5" t="n">
-        <v>24.4</v>
+        <v>23.977</v>
       </c>
       <c r="R39" s="5" t="n">
-        <v>2.44</v>
+        <v>2.398</v>
       </c>
       <c r="S39" s="6" t="inlineStr"/>
       <c r="T39" s="6" t="inlineStr">
@@ -2927,7 +2927,7 @@
       <c r="U39" s="6" t="inlineStr"/>
       <c r="V39" s="6" t="inlineStr"/>
       <c r="W39" s="5" t="n">
-        <v>24.4</v>
+        <v>23.977</v>
       </c>
     </row>
     <row r="40">
@@ -2951,7 +2951,7 @@
       <c r="H40" s="6" t="inlineStr"/>
       <c r="I40" s="6" t="inlineStr"/>
       <c r="J40" s="5" t="n">
-        <v>31.762</v>
+        <v>31.212</v>
       </c>
       <c r="K40" s="6" t="inlineStr">
         <is>
@@ -2974,16 +2974,16 @@
         </is>
       </c>
       <c r="O40" s="5" t="n">
-        <v>23.625</v>
+        <v>23.216</v>
       </c>
       <c r="P40" s="5" t="n">
-        <v>26.25</v>
+        <v>25.795</v>
       </c>
       <c r="Q40" s="5" t="n">
-        <v>26.25</v>
+        <v>25.795</v>
       </c>
       <c r="R40" s="5" t="n">
-        <v>2.625</v>
+        <v>2.58</v>
       </c>
       <c r="S40" s="6" t="inlineStr"/>
       <c r="T40" s="6" t="inlineStr">
@@ -2994,7 +2994,7 @@
       <c r="U40" s="6" t="inlineStr"/>
       <c r="V40" s="6" t="inlineStr"/>
       <c r="W40" s="5" t="n">
-        <v>26.25</v>
+        <v>25.795</v>
       </c>
     </row>
     <row r="41">
@@ -3018,7 +3018,7 @@
       <c r="H41" s="6" t="inlineStr"/>
       <c r="I41" s="6" t="inlineStr"/>
       <c r="J41" s="5" t="n">
-        <v>25.628</v>
+        <v>25.184</v>
       </c>
       <c r="K41" s="6" t="inlineStr">
         <is>
@@ -3041,16 +3041,16 @@
         </is>
       </c>
       <c r="O41" s="5" t="n">
-        <v>19.062</v>
+        <v>18.732</v>
       </c>
       <c r="P41" s="5" t="n">
-        <v>21.18</v>
+        <v>20.813</v>
       </c>
       <c r="Q41" s="5" t="n">
-        <v>21.18</v>
+        <v>20.813</v>
       </c>
       <c r="R41" s="5" t="n">
-        <v>2.118</v>
+        <v>2.081</v>
       </c>
       <c r="S41" s="6" t="inlineStr"/>
       <c r="T41" s="6" t="inlineStr">
@@ -3061,7 +3061,7 @@
       <c r="U41" s="6" t="inlineStr"/>
       <c r="V41" s="6" t="inlineStr"/>
       <c r="W41" s="5" t="n">
-        <v>21.18</v>
+        <v>20.813</v>
       </c>
     </row>
     <row r="42">
@@ -3085,7 +3085,7 @@
       <c r="H42" s="6" t="inlineStr"/>
       <c r="I42" s="6" t="inlineStr"/>
       <c r="J42" s="5" t="n">
-        <v>24.684</v>
+        <v>24.256</v>
       </c>
       <c r="K42" s="6" t="inlineStr">
         <is>
@@ -3108,16 +3108,16 @@
         </is>
       </c>
       <c r="O42" s="5" t="n">
-        <v>18.36</v>
+        <v>18.042</v>
       </c>
       <c r="P42" s="5" t="n">
-        <v>20.4</v>
+        <v>20.046</v>
       </c>
       <c r="Q42" s="5" t="n">
-        <v>20.4</v>
+        <v>20.046</v>
       </c>
       <c r="R42" s="5" t="n">
-        <v>2.04</v>
+        <v>2.005</v>
       </c>
       <c r="S42" s="6" t="inlineStr"/>
       <c r="T42" s="6" t="inlineStr">
@@ -3128,7 +3128,7 @@
       <c r="U42" s="6" t="inlineStr"/>
       <c r="V42" s="6" t="inlineStr"/>
       <c r="W42" s="5" t="n">
-        <v>20.4</v>
+        <v>20.046</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implement dynamic supplementary ratio calculation based on PL Gross Weight
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W15"/>
+  <dimension ref="A1:W39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -673,7 +673,7 @@
       <c r="H6" s="6" t="inlineStr"/>
       <c r="I6" s="6" t="inlineStr"/>
       <c r="J6" s="5" t="n">
-        <v>44.474</v>
+        <v>172.367</v>
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
@@ -692,20 +692,20 @@
       </c>
       <c r="N6" s="6" t="inlineStr">
         <is>
-          <t>SKDT/004/26-27</t>
+          <t>SKDT/002/26-27</t>
         </is>
       </c>
       <c r="O6" s="5" t="n">
-        <v>33.08</v>
+        <v>128.042</v>
       </c>
       <c r="P6" s="5" t="n">
-        <v>36.755</v>
+        <v>142.452</v>
       </c>
       <c r="Q6" s="5" t="n">
-        <v>36.755</v>
+        <v>142.452</v>
       </c>
       <c r="R6" s="5" t="n">
-        <v>3.676</v>
+        <v>14.41</v>
       </c>
       <c r="S6" s="6" t="inlineStr"/>
       <c r="T6" s="6" t="inlineStr">
@@ -716,7 +716,7 @@
       <c r="U6" s="6" t="inlineStr"/>
       <c r="V6" s="6" t="inlineStr"/>
       <c r="W6" s="5" t="n">
-        <v>36.755</v>
+        <v>142.452</v>
       </c>
     </row>
     <row r="7">
@@ -740,11 +740,11 @@
       <c r="H7" s="6" t="inlineStr"/>
       <c r="I7" s="6" t="inlineStr"/>
       <c r="J7" s="5" t="n">
-        <v>0.46</v>
+        <v>12.338</v>
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>Girls Long Sleeve Tops</t>
+          <t>Babies Long Sleeve Kimono Body</t>
         </is>
       </c>
       <c r="L7" s="6" t="inlineStr">
@@ -759,20 +759,20 @@
       </c>
       <c r="N7" s="6" t="inlineStr">
         <is>
-          <t>SKDT/004/26-27</t>
+          <t>SKDT/002/26-27</t>
         </is>
       </c>
       <c r="O7" s="5" t="n">
-        <v>0.342</v>
+        <v>9.164999999999999</v>
       </c>
       <c r="P7" s="5" t="n">
-        <v>0.379</v>
+        <v>10.196</v>
       </c>
       <c r="Q7" s="5" t="n">
-        <v>0.379</v>
+        <v>10.196</v>
       </c>
       <c r="R7" s="5" t="n">
-        <v>0.038</v>
+        <v>1.031</v>
       </c>
       <c r="S7" s="6" t="inlineStr"/>
       <c r="T7" s="6" t="inlineStr">
@@ -783,7 +783,7 @@
       <c r="U7" s="6" t="inlineStr"/>
       <c r="V7" s="6" t="inlineStr"/>
       <c r="W7" s="5" t="n">
-        <v>0.379</v>
+        <v>10.196</v>
       </c>
     </row>
     <row r="8">
@@ -807,11 +807,11 @@
       <c r="H8" s="6" t="inlineStr"/>
       <c r="I8" s="6" t="inlineStr"/>
       <c r="J8" s="5" t="n">
-        <v>53.047</v>
+        <v>29.175</v>
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
-          <t>Girls Short Sleeve Tops</t>
+          <t>Babies Long Sleeve Lapneck Body</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr">
@@ -826,20 +826,20 @@
       </c>
       <c r="N8" s="6" t="inlineStr">
         <is>
-          <t>SKDT/004/26-27</t>
+          <t>SKDT/002/26-27</t>
         </is>
       </c>
       <c r="O8" s="5" t="n">
-        <v>39.457</v>
+        <v>21.673</v>
       </c>
       <c r="P8" s="5" t="n">
-        <v>43.84</v>
+        <v>24.111</v>
       </c>
       <c r="Q8" s="5" t="n">
-        <v>43.84</v>
+        <v>24.111</v>
       </c>
       <c r="R8" s="5" t="n">
-        <v>4.384</v>
+        <v>2.439</v>
       </c>
       <c r="S8" s="6" t="inlineStr"/>
       <c r="T8" s="6" t="inlineStr">
@@ -850,7 +850,7 @@
       <c r="U8" s="6" t="inlineStr"/>
       <c r="V8" s="6" t="inlineStr"/>
       <c r="W8" s="5" t="n">
-        <v>43.84</v>
+        <v>24.111</v>
       </c>
     </row>
     <row r="9">
@@ -874,11 +874,11 @@
       <c r="H9" s="6" t="inlineStr"/>
       <c r="I9" s="6" t="inlineStr"/>
       <c r="J9" s="5" t="n">
-        <v>16.687</v>
+        <v>7.499</v>
       </c>
       <c r="K9" s="6" t="inlineStr">
         <is>
-          <t>Girls Sleeveless Suit</t>
+          <t>Babies Long Sleeve Long Leg Zip Suit</t>
         </is>
       </c>
       <c r="L9" s="6" t="inlineStr">
@@ -893,20 +893,20 @@
       </c>
       <c r="N9" s="6" t="inlineStr">
         <is>
-          <t>SKDT/004/26-27</t>
+          <t>SKDT/002/26-27</t>
         </is>
       </c>
       <c r="O9" s="5" t="n">
-        <v>12.411</v>
+        <v>5.571</v>
       </c>
       <c r="P9" s="5" t="n">
-        <v>13.79</v>
+        <v>6.197</v>
       </c>
       <c r="Q9" s="5" t="n">
-        <v>13.79</v>
+        <v>6.197</v>
       </c>
       <c r="R9" s="5" t="n">
-        <v>1.379</v>
+        <v>0.627</v>
       </c>
       <c r="S9" s="6" t="inlineStr"/>
       <c r="T9" s="6" t="inlineStr">
@@ -917,7 +917,7 @@
       <c r="U9" s="6" t="inlineStr"/>
       <c r="V9" s="6" t="inlineStr"/>
       <c r="W9" s="5" t="n">
-        <v>13.79</v>
+        <v>6.197</v>
       </c>
     </row>
     <row r="10">
@@ -941,11 +941,11 @@
       <c r="H10" s="6" t="inlineStr"/>
       <c r="I10" s="6" t="inlineStr"/>
       <c r="J10" s="5" t="n">
-        <v>38.774</v>
+        <v>29.03</v>
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>Girls Summer Sleeveless Suit</t>
+          <t>Girls Long Sleeve Long Leg Zip Suit</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr">
@@ -960,20 +960,20 @@
       </c>
       <c r="N10" s="6" t="inlineStr">
         <is>
-          <t>SKDT/004/26-27</t>
+          <t>SKDT/002/26-27</t>
         </is>
       </c>
       <c r="O10" s="5" t="n">
-        <v>28.84</v>
+        <v>21.565</v>
       </c>
       <c r="P10" s="5" t="n">
-        <v>32.044</v>
+        <v>23.991</v>
       </c>
       <c r="Q10" s="5" t="n">
-        <v>32.044</v>
+        <v>23.991</v>
       </c>
       <c r="R10" s="5" t="n">
-        <v>3.204</v>
+        <v>2.427</v>
       </c>
       <c r="S10" s="6" t="inlineStr"/>
       <c r="T10" s="6" t="inlineStr">
@@ -984,7 +984,7 @@
       <c r="U10" s="6" t="inlineStr"/>
       <c r="V10" s="6" t="inlineStr"/>
       <c r="W10" s="5" t="n">
-        <v>32.044</v>
+        <v>23.991</v>
       </c>
     </row>
     <row r="11">
@@ -1008,11 +1008,11 @@
       <c r="H11" s="6" t="inlineStr"/>
       <c r="I11" s="6" t="inlineStr"/>
       <c r="J11" s="5" t="n">
-        <v>61.506</v>
+        <v>48.674</v>
       </c>
       <c r="K11" s="6" t="inlineStr">
         <is>
-          <t>Girls Baggy Pants</t>
+          <t>Babies Short Sleeve Short Leg Suit</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
@@ -1027,20 +1027,20 @@
       </c>
       <c r="N11" s="6" t="inlineStr">
         <is>
-          <t>SKDT/004/26-27</t>
+          <t>SKDT/002/26-27</t>
         </is>
       </c>
       <c r="O11" s="5" t="n">
-        <v>45.748</v>
+        <v>36.157</v>
       </c>
       <c r="P11" s="5" t="n">
-        <v>50.831</v>
+        <v>40.226</v>
       </c>
       <c r="Q11" s="5" t="n">
-        <v>50.831</v>
+        <v>40.226</v>
       </c>
       <c r="R11" s="5" t="n">
-        <v>5.083</v>
+        <v>4.069</v>
       </c>
       <c r="S11" s="6" t="inlineStr"/>
       <c r="T11" s="6" t="inlineStr">
@@ -1051,7 +1051,7 @@
       <c r="U11" s="6" t="inlineStr"/>
       <c r="V11" s="6" t="inlineStr"/>
       <c r="W11" s="5" t="n">
-        <v>50.831</v>
+        <v>40.226</v>
       </c>
     </row>
     <row r="12">
@@ -1075,11 +1075,11 @@
       <c r="H12" s="6" t="inlineStr"/>
       <c r="I12" s="6" t="inlineStr"/>
       <c r="J12" s="5" t="n">
-        <v>43.67</v>
+        <v>14.128</v>
       </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
-          <t>Girls Short Pants</t>
+          <t>Babies Long Sleeve Tops</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
@@ -1094,20 +1094,20 @@
       </c>
       <c r="N12" s="6" t="inlineStr">
         <is>
-          <t>SKDT/004/26-27</t>
+          <t>SKDT/002/26-27</t>
         </is>
       </c>
       <c r="O12" s="5" t="n">
-        <v>32.482</v>
+        <v>10.495</v>
       </c>
       <c r="P12" s="5" t="n">
-        <v>36.09</v>
+        <v>11.676</v>
       </c>
       <c r="Q12" s="5" t="n">
-        <v>36.09</v>
+        <v>11.676</v>
       </c>
       <c r="R12" s="5" t="n">
-        <v>3.609</v>
+        <v>1.181</v>
       </c>
       <c r="S12" s="6" t="inlineStr"/>
       <c r="T12" s="6" t="inlineStr">
@@ -1118,7 +1118,7 @@
       <c r="U12" s="6" t="inlineStr"/>
       <c r="V12" s="6" t="inlineStr"/>
       <c r="W12" s="5" t="n">
-        <v>36.09</v>
+        <v>11.676</v>
       </c>
     </row>
     <row r="13">
@@ -1142,11 +1142,11 @@
       <c r="H13" s="6" t="inlineStr"/>
       <c r="I13" s="6" t="inlineStr"/>
       <c r="J13" s="5" t="n">
-        <v>1.241</v>
+        <v>109.226</v>
       </c>
       <c r="K13" s="6" t="inlineStr">
         <is>
-          <t>Girls Short Sleeve Skater Dress</t>
+          <t>Girls Long Sleeve Tops</t>
         </is>
       </c>
       <c r="L13" s="6" t="inlineStr">
@@ -1161,20 +1161,20 @@
       </c>
       <c r="N13" s="6" t="inlineStr">
         <is>
-          <t>SKDT/004/26-27</t>
+          <t>SKDT/002/26-27</t>
         </is>
       </c>
       <c r="O13" s="5" t="n">
-        <v>0.923</v>
+        <v>81.13800000000001</v>
       </c>
       <c r="P13" s="5" t="n">
-        <v>1.025</v>
+        <v>90.26900000000001</v>
       </c>
       <c r="Q13" s="5" t="n">
-        <v>1.025</v>
+        <v>90.26900000000001</v>
       </c>
       <c r="R13" s="5" t="n">
-        <v>0.103</v>
+        <v>9.132</v>
       </c>
       <c r="S13" s="6" t="inlineStr"/>
       <c r="T13" s="6" t="inlineStr">
@@ -1185,7 +1185,7 @@
       <c r="U13" s="6" t="inlineStr"/>
       <c r="V13" s="6" t="inlineStr"/>
       <c r="W13" s="5" t="n">
-        <v>1.025</v>
+        <v>90.26900000000001</v>
       </c>
     </row>
     <row r="14">
@@ -1199,7 +1199,7 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>95% ORGANIC COTTON 5% ELASTHANE KNITTED SOLID, GOTS</t>
+          <t>100% ORGANIC COTTON KNITTED INTERLOCK, GOTS PRINTED READYMADE GARMENTS</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr"/>
@@ -1209,7 +1209,7 @@
       <c r="H14" s="6" t="inlineStr"/>
       <c r="I14" s="6" t="inlineStr"/>
       <c r="J14" s="5" t="n">
-        <v>1.287</v>
+        <v>279.296</v>
       </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
@@ -1228,20 +1228,20 @@
       </c>
       <c r="N14" s="6" t="inlineStr">
         <is>
-          <t>SKDT/004/26-27</t>
+          <t>SKDT/002/26-27</t>
         </is>
       </c>
       <c r="O14" s="5" t="n">
-        <v>0.957</v>
+        <v>207.473</v>
       </c>
       <c r="P14" s="5" t="n">
-        <v>1.063</v>
+        <v>230.822</v>
       </c>
       <c r="Q14" s="5" t="n">
-        <v>1.063</v>
+        <v>230.822</v>
       </c>
       <c r="R14" s="5" t="n">
-        <v>0.106</v>
+        <v>23.35</v>
       </c>
       <c r="S14" s="6" t="inlineStr"/>
       <c r="T14" s="6" t="inlineStr">
@@ -1252,7 +1252,7 @@
       <c r="U14" s="6" t="inlineStr"/>
       <c r="V14" s="6" t="inlineStr"/>
       <c r="W14" s="5" t="n">
-        <v>1.063</v>
+        <v>230.822</v>
       </c>
     </row>
     <row r="15">
@@ -1266,7 +1266,7 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>100% ORGANIC COTTON WOVEN GOTS PRINTED READYMADE GARMENTS</t>
+          <t>100% ORGANIC COTTON KNITTED INTERLOCK, GOTS PRINTED READYMADE GARMENTS</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr"/>
@@ -1276,11 +1276,11 @@
       <c r="H15" s="6" t="inlineStr"/>
       <c r="I15" s="6" t="inlineStr"/>
       <c r="J15" s="5" t="n">
-        <v>1.448</v>
+        <v>12.338</v>
       </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t>Sun Hats</t>
+          <t>Ladies Short Sleeve Tops</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr">
@@ -1295,20 +1295,20 @@
       </c>
       <c r="N15" s="6" t="inlineStr">
         <is>
-          <t>SKDT/004/26-27</t>
+          <t>SKDT/002/26-27</t>
         </is>
       </c>
       <c r="O15" s="5" t="n">
-        <v>1.077</v>
+        <v>9.164999999999999</v>
       </c>
       <c r="P15" s="5" t="n">
-        <v>1.196</v>
+        <v>10.196</v>
       </c>
       <c r="Q15" s="5" t="n">
-        <v>1.196</v>
+        <v>10.196</v>
       </c>
       <c r="R15" s="5" t="n">
-        <v>0.12</v>
+        <v>1.031</v>
       </c>
       <c r="S15" s="6" t="inlineStr"/>
       <c r="T15" s="6" t="inlineStr">
@@ -1319,7 +1319,1615 @@
       <c r="U15" s="6" t="inlineStr"/>
       <c r="V15" s="6" t="inlineStr"/>
       <c r="W15" s="5" t="n">
-        <v>1.196</v>
+        <v>10.196</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Sri Shanmugavel Mills Private Limited Knitting Division</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>100% ORGANIC COTTON KNITTED INTERLOCK, GOTS PRINTED READYMADE GARMENTS</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr"/>
+      <c r="E16" s="6" t="inlineStr"/>
+      <c r="F16" s="6" t="inlineStr"/>
+      <c r="G16" s="6" t="inlineStr"/>
+      <c r="H16" s="6" t="inlineStr"/>
+      <c r="I16" s="6" t="inlineStr"/>
+      <c r="J16" s="5" t="n">
+        <v>115.153</v>
+      </c>
+      <c r="K16" s="6" t="inlineStr">
+        <is>
+          <t>Babies Sleeveless Suit</t>
+        </is>
+      </c>
+      <c r="L16" s="6" t="inlineStr">
+        <is>
+          <t>21.000%</t>
+        </is>
+      </c>
+      <c r="M16" s="6" t="inlineStr">
+        <is>
+          <t>M/S. AB DUNS</t>
+        </is>
+      </c>
+      <c r="N16" s="6" t="inlineStr">
+        <is>
+          <t>SKDT/002/26-27</t>
+        </is>
+      </c>
+      <c r="O16" s="5" t="n">
+        <v>85.541</v>
+      </c>
+      <c r="P16" s="5" t="n">
+        <v>95.16800000000001</v>
+      </c>
+      <c r="Q16" s="5" t="n">
+        <v>95.16800000000001</v>
+      </c>
+      <c r="R16" s="5" t="n">
+        <v>9.627000000000001</v>
+      </c>
+      <c r="S16" s="6" t="inlineStr"/>
+      <c r="T16" s="6" t="inlineStr">
+        <is>
+          <t>GOTS</t>
+        </is>
+      </c>
+      <c r="U16" s="6" t="inlineStr"/>
+      <c r="V16" s="6" t="inlineStr"/>
+      <c r="W16" s="5" t="n">
+        <v>95.16800000000001</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Sri Shanmugavel Mills Private Limited Knitting Division</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>100% ORGANIC COTTON KNITTED INTERLOCK, GOTS PRINTED READYMADE GARMENTS</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr"/>
+      <c r="E17" s="6" t="inlineStr"/>
+      <c r="F17" s="6" t="inlineStr"/>
+      <c r="G17" s="6" t="inlineStr"/>
+      <c r="H17" s="6" t="inlineStr"/>
+      <c r="I17" s="6" t="inlineStr"/>
+      <c r="J17" s="5" t="n">
+        <v>54.141</v>
+      </c>
+      <c r="K17" s="6" t="inlineStr">
+        <is>
+          <t>Girls Sleeveless Suit</t>
+        </is>
+      </c>
+      <c r="L17" s="6" t="inlineStr">
+        <is>
+          <t>21.000%</t>
+        </is>
+      </c>
+      <c r="M17" s="6" t="inlineStr">
+        <is>
+          <t>M/S. AB DUNS</t>
+        </is>
+      </c>
+      <c r="N17" s="6" t="inlineStr">
+        <is>
+          <t>SKDT/002/26-27</t>
+        </is>
+      </c>
+      <c r="O17" s="5" t="n">
+        <v>40.219</v>
+      </c>
+      <c r="P17" s="5" t="n">
+        <v>44.745</v>
+      </c>
+      <c r="Q17" s="5" t="n">
+        <v>44.745</v>
+      </c>
+      <c r="R17" s="5" t="n">
+        <v>4.526</v>
+      </c>
+      <c r="S17" s="6" t="inlineStr"/>
+      <c r="T17" s="6" t="inlineStr">
+        <is>
+          <t>GOTS</t>
+        </is>
+      </c>
+      <c r="U17" s="6" t="inlineStr"/>
+      <c r="V17" s="6" t="inlineStr"/>
+      <c r="W17" s="5" t="n">
+        <v>44.745</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Sri Shanmugavel Mills Private Limited Knitting Division</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>100% ORGANIC COTTON KNITTED INTERLOCK, GOTS PRINTED READYMADE GARMENTS</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr"/>
+      <c r="E18" s="6" t="inlineStr"/>
+      <c r="F18" s="6" t="inlineStr"/>
+      <c r="G18" s="6" t="inlineStr"/>
+      <c r="H18" s="6" t="inlineStr"/>
+      <c r="I18" s="6" t="inlineStr"/>
+      <c r="J18" s="5" t="n">
+        <v>149.071</v>
+      </c>
+      <c r="K18" s="6" t="inlineStr">
+        <is>
+          <t>Babies Summer Sleeveless Suit</t>
+        </is>
+      </c>
+      <c r="L18" s="6" t="inlineStr">
+        <is>
+          <t>21.000%</t>
+        </is>
+      </c>
+      <c r="M18" s="6" t="inlineStr">
+        <is>
+          <t>M/S. AB DUNS</t>
+        </is>
+      </c>
+      <c r="N18" s="6" t="inlineStr">
+        <is>
+          <t>SKDT/002/26-27</t>
+        </is>
+      </c>
+      <c r="O18" s="5" t="n">
+        <v>110.736</v>
+      </c>
+      <c r="P18" s="5" t="n">
+        <v>123.198</v>
+      </c>
+      <c r="Q18" s="5" t="n">
+        <v>123.198</v>
+      </c>
+      <c r="R18" s="5" t="n">
+        <v>12.463</v>
+      </c>
+      <c r="S18" s="6" t="inlineStr"/>
+      <c r="T18" s="6" t="inlineStr">
+        <is>
+          <t>GOTS</t>
+        </is>
+      </c>
+      <c r="U18" s="6" t="inlineStr"/>
+      <c r="V18" s="6" t="inlineStr"/>
+      <c r="W18" s="5" t="n">
+        <v>123.198</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Sri Shanmugavel Mills Private Limited Knitting Division</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>100% ORGANIC COTTON KNITTED INTERLOCK, GOTS PRINTED READYMADE GARMENTS</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr"/>
+      <c r="E19" s="6" t="inlineStr"/>
+      <c r="F19" s="6" t="inlineStr"/>
+      <c r="G19" s="6" t="inlineStr"/>
+      <c r="H19" s="6" t="inlineStr"/>
+      <c r="I19" s="6" t="inlineStr"/>
+      <c r="J19" s="5" t="n">
+        <v>52.327</v>
+      </c>
+      <c r="K19" s="6" t="inlineStr">
+        <is>
+          <t>Girls Summer Sleeveless Suit</t>
+        </is>
+      </c>
+      <c r="L19" s="6" t="inlineStr">
+        <is>
+          <t>21.000%</t>
+        </is>
+      </c>
+      <c r="M19" s="6" t="inlineStr">
+        <is>
+          <t>M/S. AB DUNS</t>
+        </is>
+      </c>
+      <c r="N19" s="6" t="inlineStr">
+        <is>
+          <t>SKDT/002/26-27</t>
+        </is>
+      </c>
+      <c r="O19" s="5" t="n">
+        <v>38.871</v>
+      </c>
+      <c r="P19" s="5" t="n">
+        <v>43.245</v>
+      </c>
+      <c r="Q19" s="5" t="n">
+        <v>43.245</v>
+      </c>
+      <c r="R19" s="5" t="n">
+        <v>4.375</v>
+      </c>
+      <c r="S19" s="6" t="inlineStr"/>
+      <c r="T19" s="6" t="inlineStr">
+        <is>
+          <t>GOTS</t>
+        </is>
+      </c>
+      <c r="U19" s="6" t="inlineStr"/>
+      <c r="V19" s="6" t="inlineStr"/>
+      <c r="W19" s="5" t="n">
+        <v>43.245</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Sri Shanmugavel Mills Private Limited Knitting Division</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>100% ORGANIC COTTON KNITTED INTERLOCK, GOTS PRINTED READYMADE GARMENTS</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr"/>
+      <c r="E20" s="6" t="inlineStr"/>
+      <c r="F20" s="6" t="inlineStr"/>
+      <c r="G20" s="6" t="inlineStr"/>
+      <c r="H20" s="6" t="inlineStr"/>
+      <c r="I20" s="6" t="inlineStr"/>
+      <c r="J20" s="5" t="n">
+        <v>40.159</v>
+      </c>
+      <c r="K20" s="6" t="inlineStr">
+        <is>
+          <t>Babies Baggy Pants</t>
+        </is>
+      </c>
+      <c r="L20" s="6" t="inlineStr">
+        <is>
+          <t>21.000%</t>
+        </is>
+      </c>
+      <c r="M20" s="6" t="inlineStr">
+        <is>
+          <t>M/S. AB DUNS</t>
+        </is>
+      </c>
+      <c r="N20" s="6" t="inlineStr">
+        <is>
+          <t>SKDT/002/26-27</t>
+        </is>
+      </c>
+      <c r="O20" s="5" t="n">
+        <v>29.832</v>
+      </c>
+      <c r="P20" s="5" t="n">
+        <v>33.188</v>
+      </c>
+      <c r="Q20" s="5" t="n">
+        <v>33.188</v>
+      </c>
+      <c r="R20" s="5" t="n">
+        <v>3.357</v>
+      </c>
+      <c r="S20" s="6" t="inlineStr"/>
+      <c r="T20" s="6" t="inlineStr">
+        <is>
+          <t>GOTS</t>
+        </is>
+      </c>
+      <c r="U20" s="6" t="inlineStr"/>
+      <c r="V20" s="6" t="inlineStr"/>
+      <c r="W20" s="5" t="n">
+        <v>33.188</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Sri Shanmugavel Mills Private Limited Knitting Division</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>100% ORGANIC COTTON KNITTED INTERLOCK, GOTS PRINTED READYMADE GARMENTS</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr"/>
+      <c r="E21" s="6" t="inlineStr"/>
+      <c r="F21" s="6" t="inlineStr"/>
+      <c r="G21" s="6" t="inlineStr"/>
+      <c r="H21" s="6" t="inlineStr"/>
+      <c r="I21" s="6" t="inlineStr"/>
+      <c r="J21" s="5" t="n">
+        <v>194.503</v>
+      </c>
+      <c r="K21" s="6" t="inlineStr">
+        <is>
+          <t>Girls Baggy Pants</t>
+        </is>
+      </c>
+      <c r="L21" s="6" t="inlineStr">
+        <is>
+          <t>21.000%</t>
+        </is>
+      </c>
+      <c r="M21" s="6" t="inlineStr">
+        <is>
+          <t>M/S. AB DUNS</t>
+        </is>
+      </c>
+      <c r="N21" s="6" t="inlineStr">
+        <is>
+          <t>SKDT/002/26-27</t>
+        </is>
+      </c>
+      <c r="O21" s="5" t="n">
+        <v>144.485</v>
+      </c>
+      <c r="P21" s="5" t="n">
+        <v>160.746</v>
+      </c>
+      <c r="Q21" s="5" t="n">
+        <v>160.746</v>
+      </c>
+      <c r="R21" s="5" t="n">
+        <v>16.261</v>
+      </c>
+      <c r="S21" s="6" t="inlineStr"/>
+      <c r="T21" s="6" t="inlineStr">
+        <is>
+          <t>GOTS</t>
+        </is>
+      </c>
+      <c r="U21" s="6" t="inlineStr"/>
+      <c r="V21" s="6" t="inlineStr"/>
+      <c r="W21" s="5" t="n">
+        <v>160.746</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Sri Shanmugavel Mills Private Limited Knitting Division</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>100% ORGANIC COTTON KNITTED INTERLOCK, GOTS PRINTED READYMADE GARMENTS</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr"/>
+      <c r="E22" s="6" t="inlineStr"/>
+      <c r="F22" s="6" t="inlineStr"/>
+      <c r="G22" s="6" t="inlineStr"/>
+      <c r="H22" s="6" t="inlineStr"/>
+      <c r="I22" s="6" t="inlineStr"/>
+      <c r="J22" s="5" t="n">
+        <v>21.168</v>
+      </c>
+      <c r="K22" s="6" t="inlineStr">
+        <is>
+          <t>Ladies Baggy Pants</t>
+        </is>
+      </c>
+      <c r="L22" s="6" t="inlineStr">
+        <is>
+          <t>21.000%</t>
+        </is>
+      </c>
+      <c r="M22" s="6" t="inlineStr">
+        <is>
+          <t>M/S. AB DUNS</t>
+        </is>
+      </c>
+      <c r="N22" s="6" t="inlineStr">
+        <is>
+          <t>SKDT/002/26-27</t>
+        </is>
+      </c>
+      <c r="O22" s="5" t="n">
+        <v>15.724</v>
+      </c>
+      <c r="P22" s="5" t="n">
+        <v>17.494</v>
+      </c>
+      <c r="Q22" s="5" t="n">
+        <v>17.494</v>
+      </c>
+      <c r="R22" s="5" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="S22" s="6" t="inlineStr"/>
+      <c r="T22" s="6" t="inlineStr">
+        <is>
+          <t>GOTS</t>
+        </is>
+      </c>
+      <c r="U22" s="6" t="inlineStr"/>
+      <c r="V22" s="6" t="inlineStr"/>
+      <c r="W22" s="5" t="n">
+        <v>17.494</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>Sri Shanmugavel Mills Private Limited Knitting Division</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>100% ORGANIC COTTON KNITTED INTERLOCK, GOTS PRINTED READYMADE GARMENTS</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr"/>
+      <c r="E23" s="6" t="inlineStr"/>
+      <c r="F23" s="6" t="inlineStr"/>
+      <c r="G23" s="6" t="inlineStr"/>
+      <c r="H23" s="6" t="inlineStr"/>
+      <c r="I23" s="6" t="inlineStr"/>
+      <c r="J23" s="5" t="n">
+        <v>28.063</v>
+      </c>
+      <c r="K23" s="6" t="inlineStr">
+        <is>
+          <t>Babies Short Pants</t>
+        </is>
+      </c>
+      <c r="L23" s="6" t="inlineStr">
+        <is>
+          <t>21.000%</t>
+        </is>
+      </c>
+      <c r="M23" s="6" t="inlineStr">
+        <is>
+          <t>M/S. AB DUNS</t>
+        </is>
+      </c>
+      <c r="N23" s="6" t="inlineStr">
+        <is>
+          <t>SKDT/002/26-27</t>
+        </is>
+      </c>
+      <c r="O23" s="5" t="n">
+        <v>20.846</v>
+      </c>
+      <c r="P23" s="5" t="n">
+        <v>23.192</v>
+      </c>
+      <c r="Q23" s="5" t="n">
+        <v>23.192</v>
+      </c>
+      <c r="R23" s="5" t="n">
+        <v>2.346</v>
+      </c>
+      <c r="S23" s="6" t="inlineStr"/>
+      <c r="T23" s="6" t="inlineStr">
+        <is>
+          <t>GOTS</t>
+        </is>
+      </c>
+      <c r="U23" s="6" t="inlineStr"/>
+      <c r="V23" s="6" t="inlineStr"/>
+      <c r="W23" s="5" t="n">
+        <v>23.192</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>Sri Shanmugavel Mills Private Limited Knitting Division</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>100% ORGANIC COTTON KNITTED INTERLOCK, GOTS PRINTED READYMADE GARMENTS</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr"/>
+      <c r="E24" s="6" t="inlineStr"/>
+      <c r="F24" s="6" t="inlineStr"/>
+      <c r="G24" s="6" t="inlineStr"/>
+      <c r="H24" s="6" t="inlineStr"/>
+      <c r="I24" s="6" t="inlineStr"/>
+      <c r="J24" s="5" t="n">
+        <v>108.017</v>
+      </c>
+      <c r="K24" s="6" t="inlineStr">
+        <is>
+          <t>Girls Short Pants</t>
+        </is>
+      </c>
+      <c r="L24" s="6" t="inlineStr">
+        <is>
+          <t>21.000%</t>
+        </is>
+      </c>
+      <c r="M24" s="6" t="inlineStr">
+        <is>
+          <t>M/S. AB DUNS</t>
+        </is>
+      </c>
+      <c r="N24" s="6" t="inlineStr">
+        <is>
+          <t>SKDT/002/26-27</t>
+        </is>
+      </c>
+      <c r="O24" s="5" t="n">
+        <v>80.23999999999999</v>
+      </c>
+      <c r="P24" s="5" t="n">
+        <v>89.27</v>
+      </c>
+      <c r="Q24" s="5" t="n">
+        <v>89.27</v>
+      </c>
+      <c r="R24" s="5" t="n">
+        <v>9.029999999999999</v>
+      </c>
+      <c r="S24" s="6" t="inlineStr"/>
+      <c r="T24" s="6" t="inlineStr">
+        <is>
+          <t>GOTS</t>
+        </is>
+      </c>
+      <c r="U24" s="6" t="inlineStr"/>
+      <c r="V24" s="6" t="inlineStr"/>
+      <c r="W24" s="5" t="n">
+        <v>89.27</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>Sri Shanmugavel Mills Private Limited Knitting Division</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>100% ORGANIC COTTON KNITTED INTERLOCK, GOTS PRINTED READYMADE GARMENTS</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr"/>
+      <c r="E25" s="6" t="inlineStr"/>
+      <c r="F25" s="6" t="inlineStr"/>
+      <c r="G25" s="6" t="inlineStr"/>
+      <c r="H25" s="6" t="inlineStr"/>
+      <c r="I25" s="6" t="inlineStr"/>
+      <c r="J25" s="5" t="n">
+        <v>11.685</v>
+      </c>
+      <c r="K25" s="6" t="inlineStr">
+        <is>
+          <t>Girls Long Sleeve Skater Dress</t>
+        </is>
+      </c>
+      <c r="L25" s="6" t="inlineStr">
+        <is>
+          <t>21.000%</t>
+        </is>
+      </c>
+      <c r="M25" s="6" t="inlineStr">
+        <is>
+          <t>M/S. AB DUNS</t>
+        </is>
+      </c>
+      <c r="N25" s="6" t="inlineStr">
+        <is>
+          <t>SKDT/002/26-27</t>
+        </is>
+      </c>
+      <c r="O25" s="5" t="n">
+        <v>8.68</v>
+      </c>
+      <c r="P25" s="5" t="n">
+        <v>9.656000000000001</v>
+      </c>
+      <c r="Q25" s="5" t="n">
+        <v>9.656000000000001</v>
+      </c>
+      <c r="R25" s="5" t="n">
+        <v>0.977</v>
+      </c>
+      <c r="S25" s="6" t="inlineStr"/>
+      <c r="T25" s="6" t="inlineStr">
+        <is>
+          <t>GOTS</t>
+        </is>
+      </c>
+      <c r="U25" s="6" t="inlineStr"/>
+      <c r="V25" s="6" t="inlineStr"/>
+      <c r="W25" s="5" t="n">
+        <v>9.656000000000001</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>Sri Shanmugavel Mills Private Limited Knitting Division</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>100% ORGANIC COTTON KNITTED INTERLOCK, GOTS PRINTED READYMADE GARMENTS</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr"/>
+      <c r="E26" s="6" t="inlineStr"/>
+      <c r="F26" s="6" t="inlineStr"/>
+      <c r="G26" s="6" t="inlineStr"/>
+      <c r="H26" s="6" t="inlineStr"/>
+      <c r="I26" s="6" t="inlineStr"/>
+      <c r="J26" s="5" t="n">
+        <v>119.75</v>
+      </c>
+      <c r="K26" s="6" t="inlineStr">
+        <is>
+          <t>Girls Short Sleeve Skater Dress</t>
+        </is>
+      </c>
+      <c r="L26" s="6" t="inlineStr">
+        <is>
+          <t>21.000%</t>
+        </is>
+      </c>
+      <c r="M26" s="6" t="inlineStr">
+        <is>
+          <t>M/S. AB DUNS</t>
+        </is>
+      </c>
+      <c r="N26" s="6" t="inlineStr">
+        <is>
+          <t>SKDT/002/26-27</t>
+        </is>
+      </c>
+      <c r="O26" s="5" t="n">
+        <v>88.955</v>
+      </c>
+      <c r="P26" s="5" t="n">
+        <v>98.96599999999999</v>
+      </c>
+      <c r="Q26" s="5" t="n">
+        <v>98.96599999999999</v>
+      </c>
+      <c r="R26" s="5" t="n">
+        <v>10.011</v>
+      </c>
+      <c r="S26" s="6" t="inlineStr"/>
+      <c r="T26" s="6" t="inlineStr">
+        <is>
+          <t>GOTS</t>
+        </is>
+      </c>
+      <c r="U26" s="6" t="inlineStr"/>
+      <c r="V26" s="6" t="inlineStr"/>
+      <c r="W26" s="5" t="n">
+        <v>98.96599999999999</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>Sri Shanmugavel Mills Private Limited Knitting Division</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>100% ORGANIC COTTON KNITTED INTERLOCK, GOTS PRINTED READYMADE GARMENTS</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr"/>
+      <c r="E27" s="6" t="inlineStr"/>
+      <c r="F27" s="6" t="inlineStr"/>
+      <c r="G27" s="6" t="inlineStr"/>
+      <c r="H27" s="6" t="inlineStr"/>
+      <c r="I27" s="6" t="inlineStr"/>
+      <c r="J27" s="5" t="n">
+        <v>16.031</v>
+      </c>
+      <c r="K27" s="6" t="inlineStr">
+        <is>
+          <t>Classic Baby Cap</t>
+        </is>
+      </c>
+      <c r="L27" s="6" t="inlineStr">
+        <is>
+          <t>21.000%</t>
+        </is>
+      </c>
+      <c r="M27" s="6" t="inlineStr">
+        <is>
+          <t>M/S. AB DUNS</t>
+        </is>
+      </c>
+      <c r="N27" s="6" t="inlineStr">
+        <is>
+          <t>SKDT/002/26-27</t>
+        </is>
+      </c>
+      <c r="O27" s="5" t="n">
+        <v>11.908</v>
+      </c>
+      <c r="P27" s="5" t="n">
+        <v>13.248</v>
+      </c>
+      <c r="Q27" s="5" t="n">
+        <v>13.248</v>
+      </c>
+      <c r="R27" s="5" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="S27" s="6" t="inlineStr"/>
+      <c r="T27" s="6" t="inlineStr">
+        <is>
+          <t>GOTS</t>
+        </is>
+      </c>
+      <c r="U27" s="6" t="inlineStr"/>
+      <c r="V27" s="6" t="inlineStr"/>
+      <c r="W27" s="5" t="n">
+        <v>13.248</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>Sri Shanmugavel Mills Private Limited Knitting Division</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>100% ORGANIC COTTON KNITTED INTERLOCK, GOTS PRINTED READYMADE GARMENTS</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr"/>
+      <c r="E28" s="6" t="inlineStr"/>
+      <c r="F28" s="6" t="inlineStr"/>
+      <c r="G28" s="6" t="inlineStr"/>
+      <c r="H28" s="6" t="inlineStr"/>
+      <c r="I28" s="6" t="inlineStr"/>
+      <c r="J28" s="5" t="n">
+        <v>0.484</v>
+      </c>
+      <c r="K28" s="6" t="inlineStr">
+        <is>
+          <t>Knot Hats</t>
+        </is>
+      </c>
+      <c r="L28" s="6" t="inlineStr">
+        <is>
+          <t>21.000%</t>
+        </is>
+      </c>
+      <c r="M28" s="6" t="inlineStr">
+        <is>
+          <t>M/S. AB DUNS</t>
+        </is>
+      </c>
+      <c r="N28" s="6" t="inlineStr">
+        <is>
+          <t>SKDT/002/26-27</t>
+        </is>
+      </c>
+      <c r="O28" s="5" t="n">
+        <v>0.359</v>
+      </c>
+      <c r="P28" s="5" t="n">
+        <v>0.399</v>
+      </c>
+      <c r="Q28" s="5" t="n">
+        <v>0.399</v>
+      </c>
+      <c r="R28" s="5" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="S28" s="6" t="inlineStr"/>
+      <c r="T28" s="6" t="inlineStr">
+        <is>
+          <t>GOTS</t>
+        </is>
+      </c>
+      <c r="U28" s="6" t="inlineStr"/>
+      <c r="V28" s="6" t="inlineStr"/>
+      <c r="W28" s="5" t="n">
+        <v>0.399</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>Sri Shanmugavel Mills Private Limited Knitting Division</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>100% ORGANIC COTTON KNITTED TERRY GOTS,</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr"/>
+      <c r="E29" s="6" t="inlineStr"/>
+      <c r="F29" s="6" t="inlineStr"/>
+      <c r="G29" s="6" t="inlineStr"/>
+      <c r="H29" s="6" t="inlineStr"/>
+      <c r="I29" s="6" t="inlineStr"/>
+      <c r="J29" s="5" t="n">
+        <v>30.482</v>
+      </c>
+      <c r="K29" s="6" t="inlineStr">
+        <is>
+          <t>Girls Short Pants</t>
+        </is>
+      </c>
+      <c r="L29" s="6" t="inlineStr">
+        <is>
+          <t>21.000%</t>
+        </is>
+      </c>
+      <c r="M29" s="6" t="inlineStr">
+        <is>
+          <t>M/S. AB DUNS</t>
+        </is>
+      </c>
+      <c r="N29" s="6" t="inlineStr">
+        <is>
+          <t>SKDT/002/26-27</t>
+        </is>
+      </c>
+      <c r="O29" s="5" t="n">
+        <v>22.643</v>
+      </c>
+      <c r="P29" s="5" t="n">
+        <v>25.191</v>
+      </c>
+      <c r="Q29" s="5" t="n">
+        <v>25.191</v>
+      </c>
+      <c r="R29" s="5" t="n">
+        <v>2.548</v>
+      </c>
+      <c r="S29" s="6" t="inlineStr"/>
+      <c r="T29" s="6" t="inlineStr">
+        <is>
+          <t>GOTS</t>
+        </is>
+      </c>
+      <c r="U29" s="6" t="inlineStr"/>
+      <c r="V29" s="6" t="inlineStr"/>
+      <c r="W29" s="5" t="n">
+        <v>25.191</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Sri Shanmugavel Mills Private Limited Knitting Division</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>100% ORGANIC COTTON KNITTED TERRY GOTS,</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr"/>
+      <c r="E30" s="6" t="inlineStr"/>
+      <c r="F30" s="6" t="inlineStr"/>
+      <c r="G30" s="6" t="inlineStr"/>
+      <c r="H30" s="6" t="inlineStr"/>
+      <c r="I30" s="6" t="inlineStr"/>
+      <c r="J30" s="5" t="n">
+        <v>32.961</v>
+      </c>
+      <c r="K30" s="6" t="inlineStr">
+        <is>
+          <t>Girls Pants</t>
+        </is>
+      </c>
+      <c r="L30" s="6" t="inlineStr">
+        <is>
+          <t>21.000%</t>
+        </is>
+      </c>
+      <c r="M30" s="6" t="inlineStr">
+        <is>
+          <t>M/S. AB DUNS</t>
+        </is>
+      </c>
+      <c r="N30" s="6" t="inlineStr">
+        <is>
+          <t>SKDT/002/26-27</t>
+        </is>
+      </c>
+      <c r="O30" s="5" t="n">
+        <v>24.485</v>
+      </c>
+      <c r="P30" s="5" t="n">
+        <v>27.24</v>
+      </c>
+      <c r="Q30" s="5" t="n">
+        <v>27.24</v>
+      </c>
+      <c r="R30" s="5" t="n">
+        <v>2.756</v>
+      </c>
+      <c r="S30" s="6" t="inlineStr"/>
+      <c r="T30" s="6" t="inlineStr">
+        <is>
+          <t>GOTS</t>
+        </is>
+      </c>
+      <c r="U30" s="6" t="inlineStr"/>
+      <c r="V30" s="6" t="inlineStr"/>
+      <c r="W30" s="5" t="n">
+        <v>27.24</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>Sri Shanmugavel Mills Private Limited Knitting Division</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>100% ORGANIC COTTON WOVEN GOTS PRINTED READYMADE GARMENTS</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr"/>
+      <c r="E31" s="6" t="inlineStr"/>
+      <c r="F31" s="6" t="inlineStr"/>
+      <c r="G31" s="6" t="inlineStr"/>
+      <c r="H31" s="6" t="inlineStr"/>
+      <c r="I31" s="6" t="inlineStr"/>
+      <c r="J31" s="5" t="n">
+        <v>15.241</v>
+      </c>
+      <c r="K31" s="6" t="inlineStr">
+        <is>
+          <t>Sun Hats</t>
+        </is>
+      </c>
+      <c r="L31" s="6" t="inlineStr">
+        <is>
+          <t>21.000%</t>
+        </is>
+      </c>
+      <c r="M31" s="6" t="inlineStr">
+        <is>
+          <t>M/S. AB DUNS</t>
+        </is>
+      </c>
+      <c r="N31" s="6" t="inlineStr">
+        <is>
+          <t>SKDT/002/26-27</t>
+        </is>
+      </c>
+      <c r="O31" s="5" t="n">
+        <v>11.322</v>
+      </c>
+      <c r="P31" s="5" t="n">
+        <v>12.595</v>
+      </c>
+      <c r="Q31" s="5" t="n">
+        <v>12.595</v>
+      </c>
+      <c r="R31" s="5" t="n">
+        <v>1.274</v>
+      </c>
+      <c r="S31" s="6" t="inlineStr"/>
+      <c r="T31" s="6" t="inlineStr">
+        <is>
+          <t>GOTS</t>
+        </is>
+      </c>
+      <c r="U31" s="6" t="inlineStr"/>
+      <c r="V31" s="6" t="inlineStr"/>
+      <c r="W31" s="5" t="n">
+        <v>12.595</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Sri Shanmugavel Mills Private Limited Knitting Division</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>95% ORGANIC COTTON 5% ELASTHANE KNITTED SOLID, GOTS</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr"/>
+      <c r="E32" s="6" t="inlineStr"/>
+      <c r="F32" s="6" t="inlineStr"/>
+      <c r="G32" s="6" t="inlineStr"/>
+      <c r="H32" s="6" t="inlineStr"/>
+      <c r="I32" s="6" t="inlineStr"/>
+      <c r="J32" s="5" t="n">
+        <v>1.742</v>
+      </c>
+      <c r="K32" s="6" t="inlineStr">
+        <is>
+          <t>Babies Baggy Pants</t>
+        </is>
+      </c>
+      <c r="L32" s="6" t="inlineStr">
+        <is>
+          <t>21.000%</t>
+        </is>
+      </c>
+      <c r="M32" s="6" t="inlineStr">
+        <is>
+          <t>M/S. AB DUNS</t>
+        </is>
+      </c>
+      <c r="N32" s="6" t="inlineStr">
+        <is>
+          <t>SKDT/002/26-27</t>
+        </is>
+      </c>
+      <c r="O32" s="5" t="n">
+        <v>1.294</v>
+      </c>
+      <c r="P32" s="5" t="n">
+        <v>1.439</v>
+      </c>
+      <c r="Q32" s="5" t="n">
+        <v>1.439</v>
+      </c>
+      <c r="R32" s="5" t="n">
+        <v>0.146</v>
+      </c>
+      <c r="S32" s="6" t="inlineStr"/>
+      <c r="T32" s="6" t="inlineStr">
+        <is>
+          <t>GOTS</t>
+        </is>
+      </c>
+      <c r="U32" s="6" t="inlineStr"/>
+      <c r="V32" s="6" t="inlineStr"/>
+      <c r="W32" s="5" t="n">
+        <v>1.439</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>Sri Shanmugavel Mills Private Limited Knitting Division</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>95% ORGANIC COTTON 5% ELASTHANE KNITTED SOLID, GOTS</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr"/>
+      <c r="E33" s="6" t="inlineStr"/>
+      <c r="F33" s="6" t="inlineStr"/>
+      <c r="G33" s="6" t="inlineStr"/>
+      <c r="H33" s="6" t="inlineStr"/>
+      <c r="I33" s="6" t="inlineStr"/>
+      <c r="J33" s="5" t="n">
+        <v>19.886</v>
+      </c>
+      <c r="K33" s="6" t="inlineStr">
+        <is>
+          <t>Girls Baggy Pants</t>
+        </is>
+      </c>
+      <c r="L33" s="6" t="inlineStr">
+        <is>
+          <t>21.000%</t>
+        </is>
+      </c>
+      <c r="M33" s="6" t="inlineStr">
+        <is>
+          <t>M/S. AB DUNS</t>
+        </is>
+      </c>
+      <c r="N33" s="6" t="inlineStr">
+        <is>
+          <t>SKDT/002/26-27</t>
+        </is>
+      </c>
+      <c r="O33" s="5" t="n">
+        <v>14.772</v>
+      </c>
+      <c r="P33" s="5" t="n">
+        <v>16.434</v>
+      </c>
+      <c r="Q33" s="5" t="n">
+        <v>16.434</v>
+      </c>
+      <c r="R33" s="5" t="n">
+        <v>1.662</v>
+      </c>
+      <c r="S33" s="6" t="inlineStr"/>
+      <c r="T33" s="6" t="inlineStr">
+        <is>
+          <t>GOTS</t>
+        </is>
+      </c>
+      <c r="U33" s="6" t="inlineStr"/>
+      <c r="V33" s="6" t="inlineStr"/>
+      <c r="W33" s="5" t="n">
+        <v>16.434</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="n">
+        <v>29</v>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>Sri Shanmugavel Mills Private Limited Knitting Division</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>95% ORGANIC COTTON 5% ELASTHANE KNITTED SOLID, GOTS</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr"/>
+      <c r="E34" s="6" t="inlineStr"/>
+      <c r="F34" s="6" t="inlineStr"/>
+      <c r="G34" s="6" t="inlineStr"/>
+      <c r="H34" s="6" t="inlineStr"/>
+      <c r="I34" s="6" t="inlineStr"/>
+      <c r="J34" s="5" t="n">
+        <v>2.177</v>
+      </c>
+      <c r="K34" s="6" t="inlineStr">
+        <is>
+          <t>Ladies Baggy Pants</t>
+        </is>
+      </c>
+      <c r="L34" s="6" t="inlineStr">
+        <is>
+          <t>21.000%</t>
+        </is>
+      </c>
+      <c r="M34" s="6" t="inlineStr">
+        <is>
+          <t>M/S. AB DUNS</t>
+        </is>
+      </c>
+      <c r="N34" s="6" t="inlineStr">
+        <is>
+          <t>SKDT/002/26-27</t>
+        </is>
+      </c>
+      <c r="O34" s="5" t="n">
+        <v>1.617</v>
+      </c>
+      <c r="P34" s="5" t="n">
+        <v>1.799</v>
+      </c>
+      <c r="Q34" s="5" t="n">
+        <v>1.799</v>
+      </c>
+      <c r="R34" s="5" t="n">
+        <v>0.182</v>
+      </c>
+      <c r="S34" s="6" t="inlineStr"/>
+      <c r="T34" s="6" t="inlineStr">
+        <is>
+          <t>GOTS</t>
+        </is>
+      </c>
+      <c r="U34" s="6" t="inlineStr"/>
+      <c r="V34" s="6" t="inlineStr"/>
+      <c r="W34" s="5" t="n">
+        <v>1.799</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>Sri Shanmugavel Mills Private Limited Knitting Division</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>95% ORGANIC COTTON 5% ELASTHANE KNITTED SOLID, GOTS</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr"/>
+      <c r="E35" s="6" t="inlineStr"/>
+      <c r="F35" s="6" t="inlineStr"/>
+      <c r="G35" s="6" t="inlineStr"/>
+      <c r="H35" s="6" t="inlineStr"/>
+      <c r="I35" s="6" t="inlineStr"/>
+      <c r="J35" s="5" t="n">
+        <v>14.322</v>
+      </c>
+      <c r="K35" s="6" t="inlineStr">
+        <is>
+          <t>Girls Short Pants</t>
+        </is>
+      </c>
+      <c r="L35" s="6" t="inlineStr">
+        <is>
+          <t>21.000%</t>
+        </is>
+      </c>
+      <c r="M35" s="6" t="inlineStr">
+        <is>
+          <t>M/S. AB DUNS</t>
+        </is>
+      </c>
+      <c r="N35" s="6" t="inlineStr">
+        <is>
+          <t>SKDT/002/26-27</t>
+        </is>
+      </c>
+      <c r="O35" s="5" t="n">
+        <v>10.639</v>
+      </c>
+      <c r="P35" s="5" t="n">
+        <v>11.836</v>
+      </c>
+      <c r="Q35" s="5" t="n">
+        <v>11.836</v>
+      </c>
+      <c r="R35" s="5" t="n">
+        <v>1.197</v>
+      </c>
+      <c r="S35" s="6" t="inlineStr"/>
+      <c r="T35" s="6" t="inlineStr">
+        <is>
+          <t>GOTS</t>
+        </is>
+      </c>
+      <c r="U35" s="6" t="inlineStr"/>
+      <c r="V35" s="6" t="inlineStr"/>
+      <c r="W35" s="5" t="n">
+        <v>11.836</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>Sri Shanmugavel Mills Private Limited Knitting Division</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>95% ORGANIC COTTON 5% ELASTHANE KNITTED SOLID, GOTS</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr"/>
+      <c r="E36" s="6" t="inlineStr"/>
+      <c r="F36" s="6" t="inlineStr"/>
+      <c r="G36" s="6" t="inlineStr"/>
+      <c r="H36" s="6" t="inlineStr"/>
+      <c r="I36" s="6" t="inlineStr"/>
+      <c r="J36" s="5" t="n">
+        <v>10.403</v>
+      </c>
+      <c r="K36" s="6" t="inlineStr">
+        <is>
+          <t>Girls Leggings</t>
+        </is>
+      </c>
+      <c r="L36" s="6" t="inlineStr">
+        <is>
+          <t>21.000%</t>
+        </is>
+      </c>
+      <c r="M36" s="6" t="inlineStr">
+        <is>
+          <t>M/S. AB DUNS</t>
+        </is>
+      </c>
+      <c r="N36" s="6" t="inlineStr">
+        <is>
+          <t>SKDT/002/26-27</t>
+        </is>
+      </c>
+      <c r="O36" s="5" t="n">
+        <v>7.727</v>
+      </c>
+      <c r="P36" s="5" t="n">
+        <v>8.597</v>
+      </c>
+      <c r="Q36" s="5" t="n">
+        <v>8.597</v>
+      </c>
+      <c r="R36" s="5" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="S36" s="6" t="inlineStr"/>
+      <c r="T36" s="6" t="inlineStr">
+        <is>
+          <t>GOTS</t>
+        </is>
+      </c>
+      <c r="U36" s="6" t="inlineStr"/>
+      <c r="V36" s="6" t="inlineStr"/>
+      <c r="W36" s="5" t="n">
+        <v>8.597</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>Sri Shanmugavel Mills Private Limited Knitting Division</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>95% ORGANIC COTTON 5% ELASTHANE KNITTED SOLID, GOTS</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="inlineStr"/>
+      <c r="E37" s="6" t="inlineStr"/>
+      <c r="F37" s="6" t="inlineStr"/>
+      <c r="G37" s="6" t="inlineStr"/>
+      <c r="H37" s="6" t="inlineStr"/>
+      <c r="I37" s="6" t="inlineStr"/>
+      <c r="J37" s="5" t="n">
+        <v>8.516</v>
+      </c>
+      <c r="K37" s="6" t="inlineStr">
+        <is>
+          <t>Girls Long Sleeve Tops</t>
+        </is>
+      </c>
+      <c r="L37" s="6" t="inlineStr">
+        <is>
+          <t>21.000%</t>
+        </is>
+      </c>
+      <c r="M37" s="6" t="inlineStr">
+        <is>
+          <t>M/S. AB DUNS</t>
+        </is>
+      </c>
+      <c r="N37" s="6" t="inlineStr">
+        <is>
+          <t>SKDT/002/26-27</t>
+        </is>
+      </c>
+      <c r="O37" s="5" t="n">
+        <v>6.326</v>
+      </c>
+      <c r="P37" s="5" t="n">
+        <v>7.037</v>
+      </c>
+      <c r="Q37" s="5" t="n">
+        <v>7.037</v>
+      </c>
+      <c r="R37" s="5" t="n">
+        <v>0.712</v>
+      </c>
+      <c r="S37" s="6" t="inlineStr"/>
+      <c r="T37" s="6" t="inlineStr">
+        <is>
+          <t>GOTS</t>
+        </is>
+      </c>
+      <c r="U37" s="6" t="inlineStr"/>
+      <c r="V37" s="6" t="inlineStr"/>
+      <c r="W37" s="5" t="n">
+        <v>7.037</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>Sri Shanmugavel Mills Private Limited Knitting Division</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>95% ORGANIC COTTON 5% ELASTHANE KNITTED SOLID, GOTS</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr"/>
+      <c r="E38" s="6" t="inlineStr"/>
+      <c r="F38" s="6" t="inlineStr"/>
+      <c r="G38" s="6" t="inlineStr"/>
+      <c r="H38" s="6" t="inlineStr"/>
+      <c r="I38" s="6" t="inlineStr"/>
+      <c r="J38" s="5" t="n">
+        <v>17.539</v>
+      </c>
+      <c r="K38" s="6" t="inlineStr">
+        <is>
+          <t>Girls Short Sleeve Tops</t>
+        </is>
+      </c>
+      <c r="L38" s="6" t="inlineStr">
+        <is>
+          <t>21.000%</t>
+        </is>
+      </c>
+      <c r="M38" s="6" t="inlineStr">
+        <is>
+          <t>M/S. AB DUNS</t>
+        </is>
+      </c>
+      <c r="N38" s="6" t="inlineStr">
+        <is>
+          <t>SKDT/002/26-27</t>
+        </is>
+      </c>
+      <c r="O38" s="5" t="n">
+        <v>13.029</v>
+      </c>
+      <c r="P38" s="5" t="n">
+        <v>14.495</v>
+      </c>
+      <c r="Q38" s="5" t="n">
+        <v>14.495</v>
+      </c>
+      <c r="R38" s="5" t="n">
+        <v>1.466</v>
+      </c>
+      <c r="S38" s="6" t="inlineStr"/>
+      <c r="T38" s="6" t="inlineStr">
+        <is>
+          <t>GOTS</t>
+        </is>
+      </c>
+      <c r="U38" s="6" t="inlineStr"/>
+      <c r="V38" s="6" t="inlineStr"/>
+      <c r="W38" s="5" t="n">
+        <v>14.495</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>Sri Shanmugavel Mills Private Limited Knitting Division</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>95% ORGANIC COTTON 5% ELASTHANE KNITTED SOLID, GOTS</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr"/>
+      <c r="E39" s="6" t="inlineStr"/>
+      <c r="F39" s="6" t="inlineStr"/>
+      <c r="G39" s="6" t="inlineStr"/>
+      <c r="H39" s="6" t="inlineStr"/>
+      <c r="I39" s="6" t="inlineStr"/>
+      <c r="J39" s="5" t="n">
+        <v>4.355</v>
+      </c>
+      <c r="K39" s="6" t="inlineStr">
+        <is>
+          <t>Babies Long Sleeve Lapneck Body</t>
+        </is>
+      </c>
+      <c r="L39" s="6" t="inlineStr">
+        <is>
+          <t>21.000%</t>
+        </is>
+      </c>
+      <c r="M39" s="6" t="inlineStr">
+        <is>
+          <t>M/S. AB DUNS</t>
+        </is>
+      </c>
+      <c r="N39" s="6" t="inlineStr">
+        <is>
+          <t>SKDT/002/26-27</t>
+        </is>
+      </c>
+      <c r="O39" s="5" t="n">
+        <v>3.235</v>
+      </c>
+      <c r="P39" s="5" t="n">
+        <v>3.598</v>
+      </c>
+      <c r="Q39" s="5" t="n">
+        <v>3.598</v>
+      </c>
+      <c r="R39" s="5" t="n">
+        <v>0.364</v>
+      </c>
+      <c r="S39" s="6" t="inlineStr"/>
+      <c r="T39" s="6" t="inlineStr">
+        <is>
+          <t>GOTS</t>
+        </is>
+      </c>
+      <c r="U39" s="6" t="inlineStr"/>
+      <c r="V39" s="6" t="inlineStr"/>
+      <c r="W39" s="5" t="n">
+        <v>3.598</v>
       </c>
     </row>
   </sheetData>

</xml_diff>